<commit_message>
rename images and upload to cloudinary
</commit_message>
<xml_diff>
--- a/all_workouts_final_with_descriptions3.xlsx
+++ b/all_workouts_final_with_descriptions3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UNIVERSITY\GraduationProject\MoveOn.FastAPI\WorkoutGeneration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA810668-3ECB-482D-AB08-D7FBCC43D53A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC353FBC-88C6-497B-80A6-AFB3F103D65F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -778,22 +778,29 @@
     <t>Lie flat on your back, hands under glutes, legs extended. Lift both feet a few inches off the floor — keep them there the entire set. Alternate raising and lowering each leg in short, rapid kicks — like a freestyle swimming motion. Keep lower back pressed into the floor. Breathe steadily throughout.</t>
   </si>
   <si>
-    <t xml:space="preserve"> Deadleft</t>
-  </si>
-  <si>
     <t>Dumbbell Front Raises</t>
+  </si>
+  <si>
+    <t>Deadleft</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -841,19 +848,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -1351,7 +1361,7 @@
   <dimension ref="A1:H121"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="4" max="4" width="18.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="50.109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="63.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1944,7 +1954,7 @@
         <v>1</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E26" t="s">
         <v>18</v>
@@ -3300,8 +3310,8 @@
       <c r="C85">
         <v>6</v>
       </c>
-      <c r="D85" s="4" t="s">
-        <v>252</v>
+      <c r="D85" s="5" t="s">
+        <v>253</v>
       </c>
       <c r="E85" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
add imags link to the xls file
</commit_message>
<xml_diff>
--- a/all_workouts_final_with_descriptions3.xlsx
+++ b/all_workouts_final_with_descriptions3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UNIVERSITY\GraduationProject\MoveOn.FastAPI\WorkoutGeneration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC353FBC-88C6-497B-80A6-AFB3F103D65F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D5A4DAC-EFDC-47FB-8EAD-FA8FEBA716AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="312">
   <si>
     <t>Muscle_Group</t>
   </si>
@@ -782,18 +782,199 @@
   </si>
   <si>
     <t>Deadleft</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631433/moveon/Final_Images/Tricep%20Machine%20Dip.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631432/moveon/Final_Images/T-Bar%20Rows.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Straight%20Arm%20Pulldowns.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Standing%20Calf%20Raises.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631430/moveon/Final_Images/Spider%20Curls.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631428/moveon/Final_Images/Single-Arm%20Dumbbell%20Row.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631427/moveon/Final_Images/Seated%20Rows%20Close-Grip.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631426/moveon/Final_Images/Seated%20Leg%20Curl.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631425/moveon/Final_Images/Seated%20Calf%20Raises.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631422/moveon/Final_Images/Russian%20Twists.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Rope%20Pushdowns.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Romani%20Deadleft.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631420/moveon/Final_Images/Preacher%20Curls.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631419/moveon/Final_Images/Plank.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631418/moveon/Final_Images/Pec%20Deck%20Flyes.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631418/moveon/Final_Images/Mountain%20Climbers.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631417/moveon/Final_Images/Machine%20Shoulder%20Press.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631416/moveon/Final_Images/Machine%20Bench%20Press.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631415/moveon/Final_Images/Lying%20Leg%20Curl.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631415/moveon/Final_Images/Lunges.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631413/moveon/Final_Images/Leg%20Raises.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631413/moveon/Final_Images/Leg%20Press.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631412/moveon/Final_Images/Leg%20Extensions.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631411/moveon/Final_Images/Lateral%20Raises.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631410/moveon/Final_Images/Lat%20Pulldowns.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline%20Dumbbell%20Press.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline%20Dumbbell%20Curls.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631408/moveon/Final_Images/Incline%20Barbell%20Press.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip%20Thrust.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip%20Adductor%20Machine.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631406/moveon/Final_Images/Hanging%20Knee%20Raises.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631405/moveon/Final_Images/Hack%20Squats.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631405/moveon/Final_Images/Glute%20Bridges.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631403/moveon/Final_Images/Flutter%20Kicks.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631402/moveon/Final_Images/Face%20Pulls.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631402/moveon/Final_Images/Dumbbell%20Tricep%20Kickback.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631401/moveon/Final_Images/Dumbbell%20Rows.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631400/moveon/Final_Images/Dumbbell%20Overhead%20Press.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631399/moveon/Final_Images/Dumbbell%20Front%20Raises.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631398/moveon/Final_Images/Dumbbell%20Curls.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631398/moveon/Final_Images/Dumbbell%20Bench%20Press.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631396/moveon/Final_Images/Concentration%20Curls.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631397/moveon/Final_Images/Crunches.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631395/moveon/Final_Images/close-grip-push-up.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631395/moveon/Final_Images/Close-Grip%20Bench%20Press.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631394/moveon/Final_Images/Cable%20Lateral%20Raises.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631393/moveon/Final_Images/Cable%20Curls.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631392/moveon/Final_Images/Cable%20Crossovers%20High%20to%20Low.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631392/moveon/Final_Images/Bicycle%20Crunches.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell%20Squats.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell%20Rows.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631390/moveon/Final_Images/Barbell%20Overhead%20Press.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631389/moveon/Final_Images/Barbell%20Curls.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631388/moveon/Final_Images/Barbell%20Bench%20Press.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631387/moveon/Final_Images/Ab%20Wheel%20Rollouts.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776636921/Overhead_Rope_Extensions_p2c1jc.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776637097/Single-Arm_Cable_Pushdown_dhbw3z.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776637253/cable-seated-crunch_yeatfx.webp</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -848,19 +1029,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -1361,8 +1545,14 @@
   <dimension ref="A1:H121"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="4" max="4" width="50.109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="63.6640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="18.77734375" customWidth="1"/>
+    <col min="3" max="3" width="3.109375" customWidth="1"/>
+    <col min="4" max="4" width="26.77734375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="3.21875" customWidth="1"/>
+    <col min="6" max="6" width="67.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="109.5546875" customWidth="1"/>
+    <col min="8" max="8" width="27.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1410,6 +1600,9 @@
       <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G2" s="3" t="s">
+        <v>307</v>
+      </c>
       <c r="H2" t="s">
         <v>13</v>
       </c>
@@ -1433,6 +1626,9 @@
       <c r="F3" t="s">
         <v>15</v>
       </c>
+      <c r="G3" s="3" t="s">
+        <v>281</v>
+      </c>
       <c r="H3" t="s">
         <v>16</v>
       </c>
@@ -1456,6 +1652,9 @@
       <c r="F4" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="G4" s="3" t="s">
+        <v>301</v>
+      </c>
       <c r="H4" t="s">
         <v>20</v>
       </c>
@@ -1479,6 +1678,9 @@
       <c r="F5" t="s">
         <v>23</v>
       </c>
+      <c r="G5" s="3" t="s">
+        <v>294</v>
+      </c>
       <c r="H5" t="s">
         <v>24</v>
       </c>
@@ -1502,6 +1704,9 @@
       <c r="F6" t="s">
         <v>26</v>
       </c>
+      <c r="G6" s="3" t="s">
+        <v>279</v>
+      </c>
       <c r="H6" t="s">
         <v>27</v>
       </c>
@@ -1525,6 +1730,9 @@
       <c r="F7" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="G7" s="3" t="s">
+        <v>301</v>
+      </c>
       <c r="H7" t="s">
         <v>20</v>
       </c>
@@ -1548,6 +1756,9 @@
       <c r="F8" t="s">
         <v>30</v>
       </c>
+      <c r="G8" s="3" t="s">
+        <v>271</v>
+      </c>
       <c r="H8" t="s">
         <v>31</v>
       </c>
@@ -1571,6 +1782,9 @@
       <c r="F9" t="s">
         <v>26</v>
       </c>
+      <c r="G9" s="3" t="s">
+        <v>279</v>
+      </c>
       <c r="H9" t="s">
         <v>27</v>
       </c>
@@ -1594,6 +1808,9 @@
       <c r="F10" t="s">
         <v>33</v>
       </c>
+      <c r="G10" s="3" t="s">
+        <v>254</v>
+      </c>
       <c r="H10" t="s">
         <v>34</v>
       </c>
@@ -1617,6 +1834,9 @@
       <c r="F11" t="s">
         <v>30</v>
       </c>
+      <c r="G11" s="3" t="s">
+        <v>271</v>
+      </c>
       <c r="H11" t="s">
         <v>31</v>
       </c>
@@ -1640,6 +1860,9 @@
       <c r="F12" t="s">
         <v>15</v>
       </c>
+      <c r="G12" s="3" t="s">
+        <v>281</v>
+      </c>
       <c r="H12" t="s">
         <v>16</v>
       </c>
@@ -1663,6 +1886,9 @@
       <c r="F13" t="s">
         <v>37</v>
       </c>
+      <c r="G13" s="3" t="s">
+        <v>268</v>
+      </c>
       <c r="H13" t="s">
         <v>38</v>
       </c>
@@ -1686,6 +1912,9 @@
       <c r="F14" t="s">
         <v>12</v>
       </c>
+      <c r="G14" s="3" t="s">
+        <v>307</v>
+      </c>
       <c r="H14" t="s">
         <v>13</v>
       </c>
@@ -1709,6 +1938,9 @@
       <c r="F15" t="s">
         <v>15</v>
       </c>
+      <c r="G15" s="3" t="s">
+        <v>281</v>
+      </c>
       <c r="H15" t="s">
         <v>16</v>
       </c>
@@ -1732,6 +1964,9 @@
       <c r="F16" t="s">
         <v>37</v>
       </c>
+      <c r="G16" s="3" t="s">
+        <v>268</v>
+      </c>
       <c r="H16" t="s">
         <v>38</v>
       </c>
@@ -1755,6 +1990,9 @@
       <c r="F17" t="s">
         <v>23</v>
       </c>
+      <c r="G17" s="3" t="s">
+        <v>294</v>
+      </c>
       <c r="H17" t="s">
         <v>24</v>
       </c>
@@ -1778,6 +2016,9 @@
       <c r="F18" t="s">
         <v>26</v>
       </c>
+      <c r="G18" s="3" t="s">
+        <v>279</v>
+      </c>
       <c r="H18" t="s">
         <v>27</v>
       </c>
@@ -1801,6 +2042,9 @@
       <c r="F19" t="s">
         <v>37</v>
       </c>
+      <c r="G19" s="3" t="s">
+        <v>268</v>
+      </c>
       <c r="H19" t="s">
         <v>38</v>
       </c>
@@ -1824,6 +2068,9 @@
       <c r="F20" s="1" t="s">
         <v>44</v>
       </c>
+      <c r="G20" s="3" t="s">
+        <v>305</v>
+      </c>
       <c r="H20" t="s">
         <v>45</v>
       </c>
@@ -1847,6 +2094,9 @@
       <c r="F21" t="s">
         <v>47</v>
       </c>
+      <c r="G21" s="3" t="s">
+        <v>277</v>
+      </c>
       <c r="H21" t="s">
         <v>48</v>
       </c>
@@ -1870,6 +2120,9 @@
       <c r="F22" t="s">
         <v>51</v>
       </c>
+      <c r="G22" s="3" t="s">
+        <v>291</v>
+      </c>
       <c r="H22" t="s">
         <v>52</v>
       </c>
@@ -1893,6 +2146,9 @@
       <c r="F23" s="1" t="s">
         <v>54</v>
       </c>
+      <c r="G23" s="3" t="s">
+        <v>299</v>
+      </c>
       <c r="H23" t="s">
         <v>55</v>
       </c>
@@ -1916,6 +2172,9 @@
       <c r="F24" t="s">
         <v>58</v>
       </c>
+      <c r="G24" s="3" t="s">
+        <v>270</v>
+      </c>
       <c r="H24" t="s">
         <v>59</v>
       </c>
@@ -1939,6 +2198,9 @@
       <c r="F25" t="s">
         <v>47</v>
       </c>
+      <c r="G25" s="3" t="s">
+        <v>277</v>
+      </c>
       <c r="H25" t="s">
         <v>48</v>
       </c>
@@ -1962,6 +2224,9 @@
       <c r="F26" t="s">
         <v>61</v>
       </c>
+      <c r="G26" s="3" t="s">
+        <v>292</v>
+      </c>
       <c r="H26" t="s">
         <v>62</v>
       </c>
@@ -1985,6 +2250,9 @@
       <c r="F27" s="1" t="s">
         <v>54</v>
       </c>
+      <c r="G27" s="3" t="s">
+        <v>299</v>
+      </c>
       <c r="H27" t="s">
         <v>55</v>
       </c>
@@ -2008,6 +2276,9 @@
       <c r="F28" s="1" t="s">
         <v>44</v>
       </c>
+      <c r="G28" s="3" t="s">
+        <v>305</v>
+      </c>
       <c r="H28" t="s">
         <v>45</v>
       </c>
@@ -2031,6 +2302,9 @@
       <c r="F29" s="1" t="s">
         <v>54</v>
       </c>
+      <c r="G29" s="3" t="s">
+        <v>299</v>
+      </c>
       <c r="H29" t="s">
         <v>55</v>
       </c>
@@ -2054,6 +2328,9 @@
       <c r="F30" t="s">
         <v>51</v>
       </c>
+      <c r="G30" s="3" t="s">
+        <v>291</v>
+      </c>
       <c r="H30" t="s">
         <v>52</v>
       </c>
@@ -2077,6 +2354,9 @@
       <c r="F31" t="s">
         <v>47</v>
       </c>
+      <c r="G31" s="3" t="s">
+        <v>277</v>
+      </c>
       <c r="H31" t="s">
         <v>48</v>
       </c>
@@ -2100,6 +2380,9 @@
       <c r="F32" t="s">
         <v>68</v>
       </c>
+      <c r="G32" s="3" t="s">
+        <v>260</v>
+      </c>
       <c r="H32" t="s">
         <v>69</v>
       </c>
@@ -2123,6 +2406,9 @@
       <c r="F33" t="s">
         <v>71</v>
       </c>
+      <c r="G33" s="3" t="s">
+        <v>304</v>
+      </c>
       <c r="H33" t="s">
         <v>72</v>
       </c>
@@ -2146,6 +2432,9 @@
       <c r="F34" t="s">
         <v>74</v>
       </c>
+      <c r="G34" s="3" t="s">
+        <v>278</v>
+      </c>
       <c r="H34" t="s">
         <v>75</v>
       </c>
@@ -2169,6 +2458,9 @@
       <c r="F35" t="s">
         <v>74</v>
       </c>
+      <c r="G35" s="3" t="s">
+        <v>278</v>
+      </c>
       <c r="H35" t="s">
         <v>75</v>
       </c>
@@ -2192,6 +2484,9 @@
       <c r="F36" t="s">
         <v>78</v>
       </c>
+      <c r="G36" s="3" t="s">
+        <v>290</v>
+      </c>
       <c r="H36" t="s">
         <v>79</v>
       </c>
@@ -2215,6 +2510,9 @@
       <c r="F37" t="s">
         <v>68</v>
       </c>
+      <c r="G37" s="3" t="s">
+        <v>260</v>
+      </c>
       <c r="H37" t="s">
         <v>69</v>
       </c>
@@ -2238,6 +2536,9 @@
       <c r="F38" t="s">
         <v>82</v>
       </c>
+      <c r="G38" s="3" t="s">
+        <v>259</v>
+      </c>
       <c r="H38" t="s">
         <v>83</v>
       </c>
@@ -2261,6 +2562,9 @@
       <c r="F39" t="s">
         <v>85</v>
       </c>
+      <c r="G39" s="3" t="s">
+        <v>255</v>
+      </c>
       <c r="H39" t="s">
         <v>86</v>
       </c>
@@ -2284,6 +2588,9 @@
       <c r="F40" t="s">
         <v>88</v>
       </c>
+      <c r="G40" s="3" t="s">
+        <v>256</v>
+      </c>
       <c r="H40" t="s">
         <v>89</v>
       </c>
@@ -2307,6 +2614,9 @@
       <c r="F41" t="s">
         <v>74</v>
       </c>
+      <c r="G41" s="3" t="s">
+        <v>278</v>
+      </c>
       <c r="H41" t="s">
         <v>75</v>
       </c>
@@ -2330,6 +2640,9 @@
       <c r="F42" t="s">
         <v>68</v>
       </c>
+      <c r="G42" s="3" t="s">
+        <v>260</v>
+      </c>
       <c r="H42" t="s">
         <v>69</v>
       </c>
@@ -2353,6 +2666,9 @@
       <c r="F43" s="1" t="s">
         <v>92</v>
       </c>
+      <c r="G43" s="3" t="s">
+        <v>288</v>
+      </c>
       <c r="H43" t="s">
         <v>93</v>
       </c>
@@ -2376,6 +2692,9 @@
       <c r="F44" t="s">
         <v>71</v>
       </c>
+      <c r="G44" s="3" t="s">
+        <v>304</v>
+      </c>
       <c r="H44" t="s">
         <v>72</v>
       </c>
@@ -2399,6 +2718,9 @@
       <c r="F45" t="s">
         <v>74</v>
       </c>
+      <c r="G45" s="3" t="s">
+        <v>278</v>
+      </c>
       <c r="H45" t="s">
         <v>75</v>
       </c>
@@ -2422,6 +2744,9 @@
       <c r="F46" t="s">
         <v>82</v>
       </c>
+      <c r="G46" s="3" t="s">
+        <v>259</v>
+      </c>
       <c r="H46" t="s">
         <v>83</v>
       </c>
@@ -2445,6 +2770,9 @@
       <c r="F47" t="s">
         <v>85</v>
       </c>
+      <c r="G47" s="3" t="s">
+        <v>255</v>
+      </c>
       <c r="H47" t="s">
         <v>86</v>
       </c>
@@ -2468,6 +2796,9 @@
       <c r="F48" t="s">
         <v>74</v>
       </c>
+      <c r="G48" s="3" t="s">
+        <v>278</v>
+      </c>
       <c r="H48" t="s">
         <v>75</v>
       </c>
@@ -2491,6 +2822,9 @@
       <c r="F49" t="s">
         <v>68</v>
       </c>
+      <c r="G49" s="3" t="s">
+        <v>260</v>
+      </c>
       <c r="H49" t="s">
         <v>69</v>
       </c>
@@ -2514,6 +2848,9 @@
       <c r="F50" t="s">
         <v>99</v>
       </c>
+      <c r="G50" s="3" t="s">
+        <v>306</v>
+      </c>
       <c r="H50" t="s">
         <v>100</v>
       </c>
@@ -2537,6 +2874,9 @@
       <c r="F51" t="s">
         <v>102</v>
       </c>
+      <c r="G51" s="3" t="s">
+        <v>295</v>
+      </c>
       <c r="H51" t="s">
         <v>103</v>
       </c>
@@ -2560,6 +2900,9 @@
       <c r="F52" t="s">
         <v>106</v>
       </c>
+      <c r="G52" s="3" t="s">
+        <v>293</v>
+      </c>
       <c r="H52" t="s">
         <v>107</v>
       </c>
@@ -2583,6 +2926,9 @@
       <c r="F53" t="s">
         <v>109</v>
       </c>
+      <c r="G53" s="3" t="s">
+        <v>266</v>
+      </c>
       <c r="H53" t="s">
         <v>110</v>
       </c>
@@ -2606,6 +2952,9 @@
       <c r="F54" t="s">
         <v>113</v>
       </c>
+      <c r="G54" s="3" t="s">
+        <v>300</v>
+      </c>
       <c r="H54" t="s">
         <v>114</v>
       </c>
@@ -2629,6 +2978,9 @@
       <c r="F55" t="s">
         <v>102</v>
       </c>
+      <c r="G55" s="3" t="s">
+        <v>295</v>
+      </c>
       <c r="H55" t="s">
         <v>103</v>
       </c>
@@ -2652,6 +3004,9 @@
       <c r="F56" t="s">
         <v>99</v>
       </c>
+      <c r="G56" s="3" t="s">
+        <v>306</v>
+      </c>
       <c r="H56" t="s">
         <v>100</v>
       </c>
@@ -2675,6 +3030,9 @@
       <c r="F57" t="s">
         <v>117</v>
       </c>
+      <c r="G57" s="3" t="s">
+        <v>280</v>
+      </c>
       <c r="H57" t="s">
         <v>118</v>
       </c>
@@ -2698,6 +3056,9 @@
       <c r="F58" t="s">
         <v>106</v>
       </c>
+      <c r="G58" s="3" t="s">
+        <v>293</v>
+      </c>
       <c r="H58" t="s">
         <v>107</v>
       </c>
@@ -2721,6 +3082,9 @@
       <c r="F59" t="s">
         <v>121</v>
       </c>
+      <c r="G59" s="3" t="s">
+        <v>258</v>
+      </c>
       <c r="H59" t="s">
         <v>122</v>
       </c>
@@ -2744,6 +3108,9 @@
       <c r="F60" t="s">
         <v>113</v>
       </c>
+      <c r="G60" s="3" t="s">
+        <v>300</v>
+      </c>
       <c r="H60" t="s">
         <v>114</v>
       </c>
@@ -2767,6 +3134,9 @@
       <c r="F61" t="s">
         <v>117</v>
       </c>
+      <c r="G61" s="3" t="s">
+        <v>280</v>
+      </c>
       <c r="H61" t="s">
         <v>118</v>
       </c>
@@ -2790,6 +3160,9 @@
       <c r="F62" t="s">
         <v>127</v>
       </c>
+      <c r="G62" s="3" t="s">
+        <v>289</v>
+      </c>
       <c r="H62" t="s">
         <v>128</v>
       </c>
@@ -2813,6 +3186,9 @@
       <c r="F63" t="s">
         <v>130</v>
       </c>
+      <c r="G63" s="3" t="s">
+        <v>264</v>
+      </c>
       <c r="H63" t="s">
         <v>131</v>
       </c>
@@ -2836,6 +3212,9 @@
       <c r="F64" t="s">
         <v>134</v>
       </c>
+      <c r="G64" s="3" t="s">
+        <v>254</v>
+      </c>
       <c r="H64" t="s">
         <v>135</v>
       </c>
@@ -2859,6 +3238,9 @@
       <c r="F65" t="s">
         <v>137</v>
       </c>
+      <c r="G65" s="3" t="s">
+        <v>298</v>
+      </c>
       <c r="H65" t="s">
         <v>138</v>
       </c>
@@ -2873,7 +3255,7 @@
       <c r="C66">
         <v>1</v>
       </c>
-      <c r="D66" t="s">
+      <c r="D66" s="6" t="s">
         <v>140</v>
       </c>
       <c r="E66" t="s">
@@ -2881,6 +3263,9 @@
       </c>
       <c r="F66" s="1" t="s">
         <v>141</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>310</v>
       </c>
       <c r="H66" t="s">
         <v>142</v>
@@ -2896,7 +3281,7 @@
       <c r="C67">
         <v>2</v>
       </c>
-      <c r="D67" t="s">
+      <c r="D67" s="6" t="s">
         <v>143</v>
       </c>
       <c r="E67" t="s">
@@ -2904,6 +3289,9 @@
       </c>
       <c r="F67" t="s">
         <v>130</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>264</v>
       </c>
       <c r="H67" t="s">
         <v>144</v>
@@ -2928,6 +3316,9 @@
       <c r="F68" t="s">
         <v>147</v>
       </c>
+      <c r="G68" s="3" t="s">
+        <v>309</v>
+      </c>
       <c r="H68" t="s">
         <v>148</v>
       </c>
@@ -2951,6 +3342,9 @@
       <c r="F69" t="s">
         <v>130</v>
       </c>
+      <c r="G69" s="3" t="s">
+        <v>264</v>
+      </c>
       <c r="H69" t="s">
         <v>131</v>
       </c>
@@ -2974,6 +3368,9 @@
       <c r="F70" s="1" t="s">
         <v>151</v>
       </c>
+      <c r="G70" s="3" t="s">
+        <v>289</v>
+      </c>
       <c r="H70" t="s">
         <v>152</v>
       </c>
@@ -2997,6 +3394,9 @@
       <c r="F71" t="s">
         <v>130</v>
       </c>
+      <c r="G71" s="3" t="s">
+        <v>264</v>
+      </c>
       <c r="H71" t="s">
         <v>144</v>
       </c>
@@ -3020,6 +3420,9 @@
       <c r="F72" t="s">
         <v>130</v>
       </c>
+      <c r="G72" s="3" t="s">
+        <v>264</v>
+      </c>
       <c r="H72" t="s">
         <v>131</v>
       </c>
@@ -3043,6 +3446,9 @@
       <c r="F73" t="s">
         <v>155</v>
       </c>
+      <c r="G73" s="3" t="s">
+        <v>297</v>
+      </c>
       <c r="H73" t="s">
         <v>156</v>
       </c>
@@ -3066,6 +3472,9 @@
       <c r="F74" t="s">
         <v>160</v>
       </c>
+      <c r="G74" s="3" t="s">
+        <v>275</v>
+      </c>
       <c r="H74" t="s">
         <v>161</v>
       </c>
@@ -3089,6 +3498,9 @@
       <c r="F75" t="s">
         <v>163</v>
       </c>
+      <c r="G75" s="3" t="s">
+        <v>272</v>
+      </c>
       <c r="H75" t="s">
         <v>164</v>
       </c>
@@ -3112,6 +3524,9 @@
       <c r="F76" t="s">
         <v>166</v>
       </c>
+      <c r="G76" s="3" t="s">
+        <v>283</v>
+      </c>
       <c r="H76" t="s">
         <v>167</v>
       </c>
@@ -3135,6 +3550,9 @@
       <c r="F77" s="1" t="s">
         <v>169</v>
       </c>
+      <c r="G77" s="3" t="s">
+        <v>282</v>
+      </c>
       <c r="H77" t="s">
         <v>170</v>
       </c>
@@ -3158,6 +3576,9 @@
       <c r="F78" t="s">
         <v>172</v>
       </c>
+      <c r="G78" s="3" t="s">
+        <v>257</v>
+      </c>
       <c r="H78" t="s">
         <v>173</v>
       </c>
@@ -3181,6 +3602,9 @@
       <c r="F79" s="1" t="s">
         <v>175</v>
       </c>
+      <c r="G79" s="3" t="s">
+        <v>273</v>
+      </c>
       <c r="H79" t="s">
         <v>176</v>
       </c>
@@ -3204,6 +3628,9 @@
       <c r="F80" s="1" t="s">
         <v>175</v>
       </c>
+      <c r="G80" s="3" t="s">
+        <v>273</v>
+      </c>
       <c r="H80" t="s">
         <v>179</v>
       </c>
@@ -3227,6 +3654,9 @@
       <c r="F81" t="s">
         <v>163</v>
       </c>
+      <c r="G81" s="3" t="s">
+        <v>272</v>
+      </c>
       <c r="H81" t="s">
         <v>164</v>
       </c>
@@ -3250,6 +3680,9 @@
       <c r="F82" s="1" t="s">
         <v>181</v>
       </c>
+      <c r="G82" s="3" t="s">
+        <v>276</v>
+      </c>
       <c r="H82" t="s">
         <v>182</v>
       </c>
@@ -3273,6 +3706,9 @@
       <c r="F83" t="s">
         <v>184</v>
       </c>
+      <c r="G83" s="3" t="s">
+        <v>262</v>
+      </c>
       <c r="H83" t="s">
         <v>185</v>
       </c>
@@ -3296,6 +3732,9 @@
       <c r="F84" t="s">
         <v>166</v>
       </c>
+      <c r="G84" s="3" t="s">
+        <v>283</v>
+      </c>
       <c r="H84" t="s">
         <v>167</v>
       </c>
@@ -3319,6 +3758,9 @@
       <c r="F85" t="s">
         <v>186</v>
       </c>
+      <c r="G85" s="3" t="s">
+        <v>265</v>
+      </c>
       <c r="H85" t="s">
         <v>187</v>
       </c>
@@ -3342,6 +3784,9 @@
       <c r="F86" s="1" t="s">
         <v>190</v>
       </c>
+      <c r="G86" s="3" t="s">
+        <v>285</v>
+      </c>
       <c r="H86" t="s">
         <v>191</v>
       </c>
@@ -3365,6 +3810,9 @@
       <c r="F87" t="s">
         <v>193</v>
       </c>
+      <c r="G87" s="3" t="s">
+        <v>261</v>
+      </c>
       <c r="H87" t="s">
         <v>194</v>
       </c>
@@ -3388,6 +3836,9 @@
       <c r="F88" s="1" t="s">
         <v>196</v>
       </c>
+      <c r="G88" s="3" t="s">
+        <v>286</v>
+      </c>
       <c r="H88" t="s">
         <v>197</v>
       </c>
@@ -3411,6 +3862,9 @@
       <c r="F89" t="s">
         <v>172</v>
       </c>
+      <c r="G89" s="3" t="s">
+        <v>257</v>
+      </c>
       <c r="H89" t="s">
         <v>173</v>
       </c>
@@ -3434,6 +3888,9 @@
       <c r="F90" t="s">
         <v>166</v>
       </c>
+      <c r="G90" s="3" t="s">
+        <v>283</v>
+      </c>
       <c r="H90" t="s">
         <v>167</v>
       </c>
@@ -3457,6 +3914,9 @@
       <c r="F91" s="1" t="s">
         <v>181</v>
       </c>
+      <c r="G91" s="3" t="s">
+        <v>276</v>
+      </c>
       <c r="H91" t="s">
         <v>182</v>
       </c>
@@ -3480,6 +3940,9 @@
       <c r="F92" t="s">
         <v>201</v>
       </c>
+      <c r="G92" s="3" t="s">
+        <v>303</v>
+      </c>
       <c r="H92" t="s">
         <v>202</v>
       </c>
@@ -3503,6 +3966,9 @@
       <c r="F93" t="s">
         <v>160</v>
       </c>
+      <c r="G93" s="3" t="s">
+        <v>275</v>
+      </c>
       <c r="H93" t="s">
         <v>161</v>
       </c>
@@ -3526,6 +3992,9 @@
       <c r="F94" t="s">
         <v>184</v>
       </c>
+      <c r="G94" s="3" t="s">
+        <v>261</v>
+      </c>
       <c r="H94" t="s">
         <v>194</v>
       </c>
@@ -3549,6 +4018,9 @@
       <c r="F95" t="s">
         <v>172</v>
       </c>
+      <c r="G95" s="3" t="s">
+        <v>257</v>
+      </c>
       <c r="H95" t="s">
         <v>173</v>
       </c>
@@ -3572,6 +4044,9 @@
       <c r="F96" t="s">
         <v>166</v>
       </c>
+      <c r="G96" s="3" t="s">
+        <v>283</v>
+      </c>
       <c r="H96" t="s">
         <v>167</v>
       </c>
@@ -3595,6 +4070,9 @@
       <c r="F97" s="1" t="s">
         <v>196</v>
       </c>
+      <c r="G97" s="3" t="s">
+        <v>286</v>
+      </c>
       <c r="H97" t="s">
         <v>197</v>
       </c>
@@ -3618,6 +4096,9 @@
       <c r="F98" t="s">
         <v>201</v>
       </c>
+      <c r="G98" s="3" t="s">
+        <v>303</v>
+      </c>
       <c r="H98" t="s">
         <v>202</v>
       </c>
@@ -3641,6 +4122,9 @@
       <c r="F99" s="1" t="s">
         <v>181</v>
       </c>
+      <c r="G99" s="3" t="s">
+        <v>276</v>
+      </c>
       <c r="H99" t="s">
         <v>182</v>
       </c>
@@ -3664,6 +4148,9 @@
       <c r="F100" t="s">
         <v>163</v>
       </c>
+      <c r="G100" s="3" t="s">
+        <v>272</v>
+      </c>
       <c r="H100" t="s">
         <v>164</v>
       </c>
@@ -3687,6 +4174,9 @@
       <c r="F101" t="s">
         <v>172</v>
       </c>
+      <c r="G101" s="3" t="s">
+        <v>257</v>
+      </c>
       <c r="H101" t="s">
         <v>204</v>
       </c>
@@ -3710,6 +4200,9 @@
       <c r="F102" t="s">
         <v>166</v>
       </c>
+      <c r="G102" s="3" t="s">
+        <v>283</v>
+      </c>
       <c r="H102" t="s">
         <v>167</v>
       </c>
@@ -3733,6 +4226,9 @@
       <c r="F103" t="s">
         <v>184</v>
       </c>
+      <c r="G103" s="3" t="s">
+        <v>262</v>
+      </c>
       <c r="H103" t="s">
         <v>185</v>
       </c>
@@ -3756,6 +4252,9 @@
       <c r="F104" s="1" t="s">
         <v>207</v>
       </c>
+      <c r="G104" s="3" t="s">
+        <v>303</v>
+      </c>
       <c r="H104" t="s">
         <v>208</v>
       </c>
@@ -3779,6 +4278,9 @@
       <c r="F105" s="1" t="s">
         <v>175</v>
       </c>
+      <c r="G105" s="3" t="s">
+        <v>273</v>
+      </c>
       <c r="H105" t="s">
         <v>210</v>
       </c>
@@ -3802,6 +4304,9 @@
       <c r="F106" t="s">
         <v>184</v>
       </c>
+      <c r="G106" s="3" t="s">
+        <v>261</v>
+      </c>
       <c r="H106" t="s">
         <v>194</v>
       </c>
@@ -3825,6 +4330,9 @@
       <c r="F107" t="s">
         <v>172</v>
       </c>
+      <c r="G107" s="3" t="s">
+        <v>257</v>
+      </c>
       <c r="H107" t="s">
         <v>173</v>
       </c>
@@ -3848,6 +4356,9 @@
       <c r="F108" t="s">
         <v>166</v>
       </c>
+      <c r="G108" s="3" t="s">
+        <v>283</v>
+      </c>
       <c r="H108" t="s">
         <v>167</v>
       </c>
@@ -3871,6 +4382,9 @@
       <c r="F109" s="1" t="s">
         <v>169</v>
       </c>
+      <c r="G109" s="3" t="s">
+        <v>282</v>
+      </c>
       <c r="H109" t="s">
         <v>170</v>
       </c>
@@ -3894,6 +4408,9 @@
       <c r="F110" t="s">
         <v>214</v>
       </c>
+      <c r="G110" s="3" t="s">
+        <v>296</v>
+      </c>
       <c r="H110" t="s">
         <v>215</v>
       </c>
@@ -3917,6 +4434,9 @@
       <c r="F111" s="1" t="s">
         <v>217</v>
       </c>
+      <c r="G111" s="3" t="s">
+        <v>274</v>
+      </c>
       <c r="H111" t="s">
         <v>218</v>
       </c>
@@ -3940,6 +4460,9 @@
       <c r="F112" t="s">
         <v>221</v>
       </c>
+      <c r="G112" s="3" t="s">
+        <v>267</v>
+      </c>
       <c r="H112" t="s">
         <v>222</v>
       </c>
@@ -3963,6 +4486,9 @@
       <c r="F113" s="1" t="s">
         <v>224</v>
       </c>
+      <c r="G113" s="3" t="s">
+        <v>263</v>
+      </c>
       <c r="H113" t="s">
         <v>225</v>
       </c>
@@ -3986,6 +4512,9 @@
       <c r="F114" s="1" t="s">
         <v>228</v>
       </c>
+      <c r="G114" s="3" t="s">
+        <v>311</v>
+      </c>
       <c r="H114" t="s">
         <v>229</v>
       </c>
@@ -4006,6 +4535,9 @@
       <c r="E115" t="s">
         <v>18</v>
       </c>
+      <c r="G115" s="3" t="s">
+        <v>284</v>
+      </c>
       <c r="H115" t="s">
         <v>231</v>
       </c>
@@ -4029,6 +4561,9 @@
       <c r="F116" s="1" t="s">
         <v>234</v>
       </c>
+      <c r="G116" s="3" t="s">
+        <v>269</v>
+      </c>
       <c r="H116" t="s">
         <v>235</v>
       </c>
@@ -4052,6 +4587,9 @@
       <c r="F117" s="1" t="s">
         <v>237</v>
       </c>
+      <c r="G117" s="3" t="s">
+        <v>308</v>
+      </c>
       <c r="H117" t="s">
         <v>238</v>
       </c>
@@ -4075,6 +4613,9 @@
       <c r="F118" s="3" t="s">
         <v>241</v>
       </c>
+      <c r="G118" s="3" t="s">
+        <v>274</v>
+      </c>
       <c r="H118" t="s">
         <v>242</v>
       </c>
@@ -4098,6 +4639,9 @@
       <c r="F119" s="1" t="s">
         <v>244</v>
       </c>
+      <c r="G119" s="3" t="s">
+        <v>302</v>
+      </c>
       <c r="H119" t="s">
         <v>245</v>
       </c>
@@ -4141,11 +4685,135 @@
       <c r="F121" s="1" t="s">
         <v>250</v>
       </c>
+      <c r="G121" s="3" t="s">
+        <v>287</v>
+      </c>
       <c r="H121" t="s">
         <v>251</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G10" r:id="rId1" xr:uid="{19105C44-55F9-4FCB-9097-095014F9DA3E}"/>
+    <hyperlink ref="G39" r:id="rId2" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631432/moveon/Final_Images/T-Bar Rows.webp" xr:uid="{3357DAF4-CEF1-4A2D-A618-5038B3D80DA2}"/>
+    <hyperlink ref="G40" r:id="rId3" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Straight Arm Pulldowns.webp" xr:uid="{DF101A74-11D1-4D48-A55F-70CD6E36B882}"/>
+    <hyperlink ref="G59" r:id="rId4" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631430/moveon/Final_Images/Spider Curls.webp" xr:uid="{3DB28FB9-989B-4FAB-84D8-7325E7168A51}"/>
+    <hyperlink ref="G38" r:id="rId5" xr:uid="{DDB839C0-F533-4CD6-82BA-9C7BE1D74535}"/>
+    <hyperlink ref="G42" r:id="rId6" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631427/moveon/Final_Images/Seated Rows Close-Grip.webp" xr:uid="{D84C3733-7D70-4CFF-9839-4F853A55D44D}"/>
+    <hyperlink ref="G94" r:id="rId7" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631426/moveon/Final_Images/Seated Leg Curl.webp" xr:uid="{64D59DE8-0E5D-4EA3-9A52-262F81DFB538}"/>
+    <hyperlink ref="G113" r:id="rId8" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631422/moveon/Final_Images/Russian Twists.webp" xr:uid="{97DD529F-65CB-4D95-9D52-23D3CE53F56E}"/>
+    <hyperlink ref="G63" r:id="rId9" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Rope Pushdowns.webp" xr:uid="{C5953424-AA18-47AE-A2F7-B9AFD2114352}"/>
+    <hyperlink ref="G85" r:id="rId10" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Romani Deadleft.webp" xr:uid="{AECD93F6-DA69-4D96-A009-6B5233BF04D4}"/>
+    <hyperlink ref="G53" r:id="rId11" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631420/moveon/Final_Images/Preacher Curls.webp" xr:uid="{51671F7D-7442-420A-815E-A27B5AAB5C02}"/>
+    <hyperlink ref="G112" r:id="rId12" xr:uid="{02EB4EB2-1057-4F42-B6C0-540B51CC23C0}"/>
+    <hyperlink ref="G13" r:id="rId13" xr:uid="{055FE933-E563-46DE-991F-CED9B287397A}"/>
+    <hyperlink ref="G116" r:id="rId14" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631418/moveon/Final_Images/Mountain Climbers.webp" xr:uid="{7F58DA86-9CE7-4B97-B895-8A5A94C4A5C0}"/>
+    <hyperlink ref="G24" r:id="rId15" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631417/moveon/Final_Images/Machine Shoulder Press.webp" xr:uid="{177FF476-981A-4802-8E74-D96A2EAB1E04}"/>
+    <hyperlink ref="G8" r:id="rId16" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631416/moveon/Final_Images/Machine Bench Press.webp" xr:uid="{23AE3FBD-B6FC-4F81-827E-10D6BFA8C47E}"/>
+    <hyperlink ref="G100" r:id="rId17" xr:uid="{BEC30C2A-A013-424A-B5BD-8E72787A84AD}"/>
+    <hyperlink ref="G105" r:id="rId18" xr:uid="{9E7AAEB7-6D2F-4DB1-B3A8-2A2F414BF2C1}"/>
+    <hyperlink ref="G37" r:id="rId19" xr:uid="{E4491B30-BE87-4A2D-A73F-E488D0FB7EBA}"/>
+    <hyperlink ref="G111" r:id="rId20" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631413/moveon/Final_Images/Leg Raises.webp" xr:uid="{406C5C5C-69CE-4CEA-978E-3B94865E52B4}"/>
+    <hyperlink ref="G74" r:id="rId21" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631413/moveon/Final_Images/Leg Press.webp" xr:uid="{724AC210-EEB5-46CF-B310-BEE8B9350490}"/>
+    <hyperlink ref="G82" r:id="rId22" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631412/moveon/Final_Images/Leg Extensions.webp" xr:uid="{66EBA1DB-799F-406C-84D5-6B3500581E18}"/>
+    <hyperlink ref="G21" r:id="rId23" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631411/moveon/Final_Images/Lateral Raises.webp" xr:uid="{F380D370-7BE9-4599-9D0D-4F0FC499A8A1}"/>
+    <hyperlink ref="G34" r:id="rId24" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631410/moveon/Final_Images/Lat Pulldowns.webp" xr:uid="{A77C1117-51C9-4944-981B-11FD17350623}"/>
+    <hyperlink ref="G35" r:id="rId25" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631410/moveon/Final_Images/Lat Pulldowns.webp" xr:uid="{6AEF8481-2161-4A9B-9C5A-86B3510FEBDB}"/>
+    <hyperlink ref="G6" r:id="rId26" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline Dumbbell Press.webp" xr:uid="{3DF49E4A-B9A6-4221-A806-59986067EFCA}"/>
+    <hyperlink ref="G57" r:id="rId27" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline Dumbbell Curls.webp" xr:uid="{9A524B8B-D0D9-4430-AE72-E01D0B2974C7}"/>
+    <hyperlink ref="G3" r:id="rId28" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631408/moveon/Final_Images/Incline Barbell Press.webp" xr:uid="{1B0795C6-92C3-4C25-9553-BABC3A4C5D29}"/>
+    <hyperlink ref="G109" r:id="rId29" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Thrust.webp" xr:uid="{3E2C1B7D-99E1-44DE-8499-36926F260455}"/>
+    <hyperlink ref="G102" r:id="rId30" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Adductor Machine.webp" xr:uid="{BF0D7FDE-0AB4-423D-BCA9-6293F7983A86}"/>
+    <hyperlink ref="G108" r:id="rId31" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Adductor Machine.webp" xr:uid="{6F3A60A1-1B14-481E-A73E-9C5436E7310D}"/>
+    <hyperlink ref="G115" r:id="rId32" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631406/moveon/Final_Images/Hanging Knee Raises.webp" xr:uid="{E12AABA4-A146-4865-A680-15E6F9EA667B}"/>
+    <hyperlink ref="G86" r:id="rId33" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631405/moveon/Final_Images/Hack Squats.webp" xr:uid="{152783E0-4E0D-4990-AC04-8971CEB21A9F}"/>
+    <hyperlink ref="G97" r:id="rId34" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631405/moveon/Final_Images/Glute Bridges.webp" xr:uid="{9B314E4A-043A-474E-A39C-2CC5E4C916F4}"/>
+    <hyperlink ref="G121" r:id="rId35" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631403/moveon/Final_Images/Flutter Kicks.webp" xr:uid="{A6A2F371-2ABE-4357-AB9B-1696E3F5E757}"/>
+    <hyperlink ref="G43" r:id="rId36" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631402/moveon/Final_Images/Face Pulls.webp" xr:uid="{22654AD9-6C0B-4113-9628-8246E7345A20}"/>
+    <hyperlink ref="G62" r:id="rId37" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631402/moveon/Final_Images/Dumbbell Tricep Kickback.webp" xr:uid="{00C36918-7540-4107-A53A-5A837130F0D4}"/>
+    <hyperlink ref="G36" r:id="rId38" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631401/moveon/Final_Images/Dumbbell Rows.webp" xr:uid="{0C753DF4-09A9-4B03-920E-849D848F462A}"/>
+    <hyperlink ref="G22" r:id="rId39" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631400/moveon/Final_Images/Dumbbell Overhead Press.webp" xr:uid="{316F5ACB-5893-4A79-9F87-FA14CA93FE30}"/>
+    <hyperlink ref="G26" r:id="rId40" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631399/moveon/Final_Images/Dumbbell Front Raises.webp" xr:uid="{044B8EE7-F039-4487-8023-834AD7C1246D}"/>
+    <hyperlink ref="G52" r:id="rId41" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631398/moveon/Final_Images/Dumbbell Curls.webp" xr:uid="{5ADF9132-C856-4C83-978E-67D48D4AC5A2}"/>
+    <hyperlink ref="G5" r:id="rId42" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631398/moveon/Final_Images/Dumbbell Bench Press.webp" xr:uid="{221C1554-894C-42DD-BA7C-24A1D253C005}"/>
+    <hyperlink ref="G51" r:id="rId43" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631396/moveon/Final_Images/Concentration Curls.webp" xr:uid="{D68DE0C3-B0BF-4332-9EC9-45D32B77AA1C}"/>
+    <hyperlink ref="G110" r:id="rId44" xr:uid="{4E8B250D-0E32-4383-BADC-3429C7B0B4EC}"/>
+    <hyperlink ref="G73" r:id="rId45" xr:uid="{B3ACAA6A-7137-4CA7-A2F5-46205CE6CFC8}"/>
+    <hyperlink ref="G65" r:id="rId46" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631395/moveon/Final_Images/Close-Grip Bench Press.webp" xr:uid="{D4FA6B07-0990-49AA-9601-9806EE2869FF}"/>
+    <hyperlink ref="G27" r:id="rId47" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631394/moveon/Final_Images/Cable Lateral Raises.webp" xr:uid="{A6B189E5-A81D-495F-B571-69B59D51DCAB}"/>
+    <hyperlink ref="G54" r:id="rId48" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631393/moveon/Final_Images/Cable Curls.webp" xr:uid="{E4CABCAC-C0DC-491B-A1D6-135EA36263F8}"/>
+    <hyperlink ref="G4" r:id="rId49" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631392/moveon/Final_Images/Cable Crossovers High to Low.webp" xr:uid="{50D44733-022A-41E3-A737-73DD9F3B7F0C}"/>
+    <hyperlink ref="G119" r:id="rId50" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631392/moveon/Final_Images/Bicycle Crunches.webp" xr:uid="{C2904B5E-3C9D-4CEC-8B7B-E2325905471A}"/>
+    <hyperlink ref="G92" r:id="rId51" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell Squats.webp" xr:uid="{BFF8B31F-67C3-460C-80A5-AAEF2F0BA911}"/>
+    <hyperlink ref="G33" r:id="rId52" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell Rows.webp" xr:uid="{FCC625F9-46E2-4399-A404-AED539CB8700}"/>
+    <hyperlink ref="G20" r:id="rId53" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631390/moveon/Final_Images/Barbell Overhead Press.webp" xr:uid="{54BC23DE-406D-4B96-87F3-D1DE83BDB059}"/>
+    <hyperlink ref="G50" r:id="rId54" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631389/moveon/Final_Images/Barbell Curls.webp" xr:uid="{1C564B66-22F8-4374-8D4F-AE01309211B1}"/>
+    <hyperlink ref="G2" r:id="rId55" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631388/moveon/Final_Images/Barbell Bench Press.webp" xr:uid="{5982C014-79E2-4A41-BFCD-49EC560F3613}"/>
+    <hyperlink ref="G117" r:id="rId56" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631387/moveon/Final_Images/Ab Wheel Rollouts.webp" xr:uid="{6255A00E-FA00-4393-AFD8-3CBF85A1DB7D}"/>
+    <hyperlink ref="G7" r:id="rId57" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631392/moveon/Final_Images/Cable Crossovers High to Low.webp" xr:uid="{88C66FAC-C3CE-4EEB-8E30-90D4CA3E72DF}"/>
+    <hyperlink ref="G14" r:id="rId58" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631388/moveon/Final_Images/Barbell Bench Press.webp" xr:uid="{CCC14FC3-05A0-4FE3-B7A1-6154F59D55D6}"/>
+    <hyperlink ref="G12" r:id="rId59" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631408/moveon/Final_Images/Incline Barbell Press.webp" xr:uid="{33B87BF1-6B67-4CA3-8197-A9A776E9086F}"/>
+    <hyperlink ref="G15" r:id="rId60" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631408/moveon/Final_Images/Incline Barbell Press.webp" xr:uid="{EE816864-75C5-4CA4-A517-639316DECAF1}"/>
+    <hyperlink ref="G17" r:id="rId61" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631398/moveon/Final_Images/Dumbbell Bench Press.webp" xr:uid="{C424288C-7FDF-488D-829E-1465057B85A4}"/>
+    <hyperlink ref="G11" r:id="rId62" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631416/moveon/Final_Images/Machine Bench Press.webp" xr:uid="{94A8A25E-E17F-4126-A006-DC5B52F82C4B}"/>
+    <hyperlink ref="G9" r:id="rId63" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline Dumbbell Press.webp" xr:uid="{F02B9F25-2435-4A0E-B1D7-79C438C9B06B}"/>
+    <hyperlink ref="G16" r:id="rId64" xr:uid="{4D3D7069-344C-45A1-BA0F-85C18AC6AF01}"/>
+    <hyperlink ref="G18" r:id="rId65" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline Dumbbell Press.webp" xr:uid="{9DA52350-ED9A-4EF0-8D02-735CEAE6526A}"/>
+    <hyperlink ref="G19" r:id="rId66" xr:uid="{0096A054-6DC3-41AE-B284-894E506F0BBA}"/>
+    <hyperlink ref="G23" r:id="rId67" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631394/moveon/Final_Images/Cable Lateral Raises.webp" xr:uid="{06D1FF1C-05AD-497A-B534-19D2AD82B830}"/>
+    <hyperlink ref="G25" r:id="rId68" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631411/moveon/Final_Images/Lateral Raises.webp" xr:uid="{17F90E89-40E1-4697-AC03-D72585511FAC}"/>
+    <hyperlink ref="G31" r:id="rId69" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631411/moveon/Final_Images/Lateral Raises.webp" xr:uid="{F8671347-4C54-40CD-B948-29D2F10A61FB}"/>
+    <hyperlink ref="G28" r:id="rId70" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631390/moveon/Final_Images/Barbell Overhead Press.webp" xr:uid="{FA7CFD3D-A5CA-4E43-9082-A03916DA7967}"/>
+    <hyperlink ref="G29" r:id="rId71" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631394/moveon/Final_Images/Cable Lateral Raises.webp" xr:uid="{06FFE01E-495D-4DC7-B148-9C40681E3619}"/>
+    <hyperlink ref="G30" r:id="rId72" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631400/moveon/Final_Images/Dumbbell Overhead Press.webp" xr:uid="{12EC6382-0ED3-4D62-B7D2-5B31B4A9683D}"/>
+    <hyperlink ref="G32" r:id="rId73" xr:uid="{C92111B9-BB20-495D-9C1B-0D648B62A737}"/>
+    <hyperlink ref="G41" r:id="rId74" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631410/moveon/Final_Images/Lat Pulldowns.webp" xr:uid="{ABBE89A4-9DAB-4338-93E9-03E494A93099}"/>
+    <hyperlink ref="G44" r:id="rId75" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell Rows.webp" xr:uid="{9C959A87-1031-480F-BBA1-778F3612B775}"/>
+    <hyperlink ref="G45" r:id="rId76" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631410/moveon/Final_Images/Lat Pulldowns.webp" xr:uid="{10E58E78-D714-4C6B-81B9-08DD260AEA66}"/>
+    <hyperlink ref="G48" r:id="rId77" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631410/moveon/Final_Images/Lat Pulldowns.webp" xr:uid="{E44A6EDD-EA97-4098-BB8C-4CF43CD40740}"/>
+    <hyperlink ref="G47" r:id="rId78" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631432/moveon/Final_Images/T-Bar Rows.webp" xr:uid="{3C5452B7-2202-4141-9C7A-EC33956810F0}"/>
+    <hyperlink ref="G46" r:id="rId79" xr:uid="{4CD82E2F-A252-445D-9451-8010FD9AD6EB}"/>
+    <hyperlink ref="G49" r:id="rId80" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631427/moveon/Final_Images/Seated Rows Close-Grip.webp" xr:uid="{223B65D7-1449-4DD7-B9F2-5B4A85D2792A}"/>
+    <hyperlink ref="G55" r:id="rId81" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631396/moveon/Final_Images/Concentration Curls.webp" xr:uid="{D01A618E-9222-4F1B-BDF9-091D4164FE77}"/>
+    <hyperlink ref="G56" r:id="rId82" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631389/moveon/Final_Images/Barbell Curls.webp" xr:uid="{50C5EAA6-54A2-4619-8B02-4EDE5AE521AC}"/>
+    <hyperlink ref="G58" r:id="rId83" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631398/moveon/Final_Images/Dumbbell Curls.webp" xr:uid="{39F84755-0259-4DD2-A9FB-D5FEEB83F2EF}"/>
+    <hyperlink ref="G60" r:id="rId84" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631393/moveon/Final_Images/Cable Curls.webp" xr:uid="{F68F2907-CE9C-4ECA-9FED-A239161D66B3}"/>
+    <hyperlink ref="G61" r:id="rId85" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline Dumbbell Curls.webp" xr:uid="{BF6FF696-FF4B-4449-B059-DF08605B4E9D}"/>
+    <hyperlink ref="G64" r:id="rId86" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631433/moveon/Final_Images/Tricep Machine Dip.webp" xr:uid="{AAEA9C6E-5DC5-4D74-9BDF-1FD67822FB35}"/>
+    <hyperlink ref="G69" r:id="rId87" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Rope Pushdowns.webp" xr:uid="{6DCA3703-9DCB-4D07-A0DF-C5D6828151C1}"/>
+    <hyperlink ref="G67" r:id="rId88" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Rope Pushdowns.webp" xr:uid="{46888948-A061-45DC-9F36-DC854A407B92}"/>
+    <hyperlink ref="G71" r:id="rId89" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Rope Pushdowns.webp" xr:uid="{3766BADD-6273-4970-965F-F2BBFF233855}"/>
+    <hyperlink ref="G72" r:id="rId90" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Rope Pushdowns.webp" xr:uid="{D3C98117-CE42-42A8-B023-2486311396A5}"/>
+    <hyperlink ref="G70" r:id="rId91" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631402/moveon/Final_Images/Dumbbell Tricep Kickback.webp" xr:uid="{5BFA3DE4-9F6D-4BB2-9A1C-5646F8ADE08F}"/>
+    <hyperlink ref="G75" r:id="rId92" xr:uid="{CF4B0320-ADA8-420C-B1C7-459454CB895C}"/>
+    <hyperlink ref="G81" r:id="rId93" xr:uid="{32A749A6-5A70-42B7-9970-CD158C6EE12F}"/>
+    <hyperlink ref="G76" r:id="rId94" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Adductor Machine.webp" xr:uid="{82D2A989-3FC2-49D9-8000-6FB1D1A84AB4}"/>
+    <hyperlink ref="G84" r:id="rId95" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Adductor Machine.webp" xr:uid="{C58B437B-0EA4-46B6-9B12-CE23F2ED7B9C}"/>
+    <hyperlink ref="G90" r:id="rId96" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Adductor Machine.webp" xr:uid="{D948C05A-A122-4E03-9789-57995A381430}"/>
+    <hyperlink ref="G77" r:id="rId97" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Thrust.webp" xr:uid="{221E6130-A9FF-4CE4-9E55-CD3409030E03}"/>
+    <hyperlink ref="G79" r:id="rId98" xr:uid="{7E314C35-C621-4D8A-AF50-0114F3A8AF41}"/>
+    <hyperlink ref="G80" r:id="rId99" xr:uid="{056A179E-C105-4E4E-BB74-9B83D57BDD4F}"/>
+    <hyperlink ref="G83" r:id="rId100" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631425/moveon/Final_Images/Seated Calf Raises.webp" xr:uid="{5E3148BE-8470-47E0-9EAF-04E2CC42377E}"/>
+    <hyperlink ref="G103" r:id="rId101" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631425/moveon/Final_Images/Seated Calf Raises.webp" xr:uid="{3B1903B4-0C3B-4A80-84C9-703D16670551}"/>
+    <hyperlink ref="G78" r:id="rId102" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Standing Calf Raises.webp" xr:uid="{8002D114-BE0B-437F-853C-CE2C1BCDD0ED}"/>
+    <hyperlink ref="G89" r:id="rId103" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Standing Calf Raises.webp" xr:uid="{FA5F2AA2-0574-4639-BC66-82815F98AB29}"/>
+    <hyperlink ref="G107" r:id="rId104" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Standing Calf Raises.webp" xr:uid="{FD242973-F1A5-47EC-8E91-CAA2832DD262}"/>
+    <hyperlink ref="G101" r:id="rId105" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Standing Calf Raises.webp" xr:uid="{3E1DE197-6DF5-487E-BA4D-D10A65ABDB4D}"/>
+    <hyperlink ref="G95" r:id="rId106" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Standing Calf Raises.webp" xr:uid="{0E89C214-C3C8-4F7F-9D03-2AB8FE0B41B1}"/>
+    <hyperlink ref="G87" r:id="rId107" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631426/moveon/Final_Images/Seated Leg Curl.webp" xr:uid="{400EA336-8AE2-4883-97DC-0F6D7786B52C}"/>
+    <hyperlink ref="G106" r:id="rId108" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631426/moveon/Final_Images/Seated Leg Curl.webp" xr:uid="{A77F8C5B-4FBB-4DD5-89FD-DF0C8A9DFE2E}"/>
+    <hyperlink ref="G96" r:id="rId109" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Adductor Machine.webp" xr:uid="{6D69030B-D4B1-42A6-BCC0-B66BA24AFE90}"/>
+    <hyperlink ref="G88" r:id="rId110" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631405/moveon/Final_Images/Glute Bridges.webp" xr:uid="{5906C52A-6594-4AAA-8BDE-FEA734C4737B}"/>
+    <hyperlink ref="G99" r:id="rId111" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631412/moveon/Final_Images/Leg Extensions.webp" xr:uid="{77F4402C-BF41-4B51-B987-36870A5AA104}"/>
+    <hyperlink ref="G91" r:id="rId112" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631412/moveon/Final_Images/Leg Extensions.webp" xr:uid="{43130B2B-EDE6-4A5D-A9BA-0D61FA3C00DE}"/>
+    <hyperlink ref="G98" r:id="rId113" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell Squats.webp" xr:uid="{FC3B1F98-6D43-42AF-B735-DFD505C473AC}"/>
+    <hyperlink ref="G104" r:id="rId114" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell Squats.webp" xr:uid="{319E84B5-F879-4D8A-8626-25EFC478FA27}"/>
+    <hyperlink ref="G93" r:id="rId115" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631413/moveon/Final_Images/Leg Press.webp" xr:uid="{70F9F748-B380-48FB-AC6D-0F1137622CB1}"/>
+    <hyperlink ref="G118" r:id="rId116" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631413/moveon/Final_Images/Leg Raises.webp" xr:uid="{6312C8BB-8557-47E1-A146-ADF49B132BCA}"/>
+    <hyperlink ref="G68" r:id="rId117" xr:uid="{7B36061E-64DF-40F6-9224-B944D441EEE0}"/>
+    <hyperlink ref="G66" r:id="rId118" xr:uid="{642167EC-498A-4DCF-A191-D5E1DD6CD8B2}"/>
+    <hyperlink ref="G114" r:id="rId119" xr:uid="{2DB98109-2989-4E10-B133-D04FC2208178}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
change image extination to .png
</commit_message>
<xml_diff>
--- a/all_workouts_final_with_descriptions3.xlsx
+++ b/all_workouts_final_with_descriptions3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UNIVERSITY\GraduationProject\MoveOn.FastAPI\WorkoutGeneration\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UNIVERSITY\GraduationProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D5A4DAC-EFDC-47FB-8EAD-FA8FEBA716AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2DC658EA-FF7E-40E7-ADD1-B82BE16DF709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7632" yWindow="0" windowWidth="15408" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="all_workouts_final" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="310">
   <si>
     <t>Muscle_Group</t>
   </si>
@@ -205,6 +205,9 @@
     <t>Shoulder_Variation_4</t>
   </si>
   <si>
+    <t>Front Raises</t>
+  </si>
+  <si>
     <t>https://youtu.be/tHk1sAMUcdQ?list=PLBsxOvdGIjiIQU28dc4J7zF5GnXWV7UcO</t>
   </si>
   <si>
@@ -580,6 +583,9 @@
     <t>Sit on the seated calf raise machine with pads on lower thighs, balls of feet on the platform. Lower heels as far as possible to stretch the calves — pause at the bottom. Rise up onto tiptoes as high as possible, squeeze, then lower slowly. Targets the soleus (deeper calf muscle) more than standing raises.</t>
   </si>
   <si>
+    <t>Romani Deadleft</t>
+  </si>
+  <si>
     <t>https://youtu.be/9VL38Xq8qPo?list=PLBsxOvdGIjiIl_bz4EqARJtHATATlHu1E</t>
   </si>
   <si>
@@ -763,12 +769,6 @@
     <t>Abs_Variation_6</t>
   </si>
   <si>
-    <t>Toe Touches</t>
-  </si>
-  <si>
-    <t>Lie on your back with legs raised straight up to vertical. Reach both hands up toward your toes, crunching your upper back off the floor. Try to touch your toes — the higher you reach, the harder the crunch. Lower your shoulders back down with control and repeat.</t>
-  </si>
-  <si>
     <t>Flutter Kicks</t>
   </si>
   <si>
@@ -778,217 +778,190 @@
     <t>Lie flat on your back, hands under glutes, legs extended. Lift both feet a few inches off the floor — keep them there the entire set. Alternate raising and lowering each leg in short, rapid kicks — like a freestyle swimming motion. Keep lower back pressed into the floor. Breathe steadily throughout.</t>
   </si>
   <si>
-    <t>Dumbbell Front Raises</t>
-  </si>
-  <si>
-    <t>Deadleft</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631433/moveon/Final_Images/Tricep%20Machine%20Dip.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631432/moveon/Final_Images/T-Bar%20Rows.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Straight%20Arm%20Pulldowns.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Standing%20Calf%20Raises.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631430/moveon/Final_Images/Spider%20Curls.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631428/moveon/Final_Images/Single-Arm%20Dumbbell%20Row.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631427/moveon/Final_Images/Seated%20Rows%20Close-Grip.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631426/moveon/Final_Images/Seated%20Leg%20Curl.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631425/moveon/Final_Images/Seated%20Calf%20Raises.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631422/moveon/Final_Images/Russian%20Twists.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Rope%20Pushdowns.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Romani%20Deadleft.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631420/moveon/Final_Images/Preacher%20Curls.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631419/moveon/Final_Images/Plank.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631418/moveon/Final_Images/Pec%20Deck%20Flyes.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631418/moveon/Final_Images/Mountain%20Climbers.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631417/moveon/Final_Images/Machine%20Shoulder%20Press.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631416/moveon/Final_Images/Machine%20Bench%20Press.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631415/moveon/Final_Images/Lying%20Leg%20Curl.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631415/moveon/Final_Images/Lunges.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631413/moveon/Final_Images/Leg%20Raises.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631413/moveon/Final_Images/Leg%20Press.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631412/moveon/Final_Images/Leg%20Extensions.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631411/moveon/Final_Images/Lateral%20Raises.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631410/moveon/Final_Images/Lat%20Pulldowns.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline%20Dumbbell%20Press.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline%20Dumbbell%20Curls.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631408/moveon/Final_Images/Incline%20Barbell%20Press.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip%20Thrust.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip%20Adductor%20Machine.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631406/moveon/Final_Images/Hanging%20Knee%20Raises.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631405/moveon/Final_Images/Hack%20Squats.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631405/moveon/Final_Images/Glute%20Bridges.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631403/moveon/Final_Images/Flutter%20Kicks.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631402/moveon/Final_Images/Face%20Pulls.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631402/moveon/Final_Images/Dumbbell%20Tricep%20Kickback.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631401/moveon/Final_Images/Dumbbell%20Rows.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631400/moveon/Final_Images/Dumbbell%20Overhead%20Press.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631399/moveon/Final_Images/Dumbbell%20Front%20Raises.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631398/moveon/Final_Images/Dumbbell%20Curls.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631398/moveon/Final_Images/Dumbbell%20Bench%20Press.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631396/moveon/Final_Images/Concentration%20Curls.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631397/moveon/Final_Images/Crunches.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631395/moveon/Final_Images/close-grip-push-up.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631395/moveon/Final_Images/Close-Grip%20Bench%20Press.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631394/moveon/Final_Images/Cable%20Lateral%20Raises.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631393/moveon/Final_Images/Cable%20Curls.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631392/moveon/Final_Images/Cable%20Crossovers%20High%20to%20Low.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631392/moveon/Final_Images/Bicycle%20Crunches.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell%20Squats.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell%20Rows.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631390/moveon/Final_Images/Barbell%20Overhead%20Press.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631389/moveon/Final_Images/Barbell%20Curls.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631388/moveon/Final_Images/Barbell%20Bench%20Press.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776631387/moveon/Final_Images/Ab%20Wheel%20Rollouts.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776636921/Overhead_Rope_Extensions_p2c1jc.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776637097/Single-Arm_Cable_Pushdown_dhbw3z.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776637253/cable-seated-crunch_yeatfx.webp</t>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696627/Incline_Barbell_Press_qhreoh.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696626/Incline_Dumbbell_Press_frveg3.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696618/Dumbbell_Overhead_Press_xdrupu.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696621/Face_Pulls_spwc72.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696616/Dumbbell_Bench_Press_krgpqg.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696612/Close-Grip_Bench_Press_mluyvx.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696612/Cable_Lateral_Raises_xqekaf.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696604/Barbell_Squats_cuwtbw.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696603/Ab_Wheel_Rollouts_lnzozd.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696638/Seated_Leg_Curl_s6og6e.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696637/Tricep_Machine_Dip_dgya6t.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696637/T-Bar_Rows_dcmeq9.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696637/Pec_Deck_Flyes_z7cyrn.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696637/Spider_Curls_rsb8uf.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696637/Straight_Arm_Pulldowns_no98gw.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696635/Single-Arm_Dumbbell_Row_bvkhxf.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696634/Single-Arm_Cable_Pushdown_nezyys.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696634/Seated_Rows_Close-Grip_zbdlgd.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696633/Preacher_Curls_hqawwt.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696632/Machine_Shoulder_Press_frirau.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696632/Rope_Pushdowns_zuyhpc.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696632/Overhead_Rope_Extensions_fyp2kw.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696631/Machine_Bench_Press_c6h8gz.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696628/Incline_Dumbbell_Curls_q8se8t.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696628/Lateral_Raises_cjz8qp.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696627/Lat_Pulldowns_d0xumq.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696620/Dumbbell_Front_Raises_e9urpi.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696620/Dumbbell_Tricep_Kickback_icifrk.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696619/Dumbbell_Rows_bqhz5j.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696617/Dumbbell_Curls_icudtr.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696615/close-grip-push-up_vqpfdy.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696614/Concentration_Curls_j1bxu5.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696607/Barbell_Bench_Press_mae7kd.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696611/Barbell_Rows_n32grx.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696610/Cable_Curls_as7vhi.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696609/Barbell_Curls_ixb9n2.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696607/Barbell_Overhead_Press_gqzkni.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696606/Cable_Crossovers_High_to_Low_slhpht.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696605/Bicycle_Crunches_yfq3lx.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696612/cable-seated-crunch_or9mfi.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696615/Crunches_rkzzow.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696622/Glute_Bridges_lbbnzw.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696623/Flutter_Kicks_jedpxg.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696624/Hack_Squats_zotoxt.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696625/Hanging_Knee_Raises_npgwdq.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696626/Hip_Thrust_bjmxki.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696628/Leg_Press_tvlzoe.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696628/Leg_Raises_ip1tf8.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696628/Hip_Adductor_Machine_cd40rb.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696630/Leg_Extensions_a6cays.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696630/Lunges_xgvyxq.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696630/Lying_Leg_Curl_eierha.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696631/Mountain_Climbers_clyn6t.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696631/Plank_exeuhi.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696632/Romani_Deadleft_p9bbfz.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696633/Russian_Twists_qg8b97.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696635/Seated_Calf_Raises_xlhitb.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/duprntyar/image/upload/v1776696636/Standing_Calf_Raises_dfwgbt.png</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="6">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1029,28 +1002,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1542,17 +1506,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="18.77734375" customWidth="1"/>
-    <col min="3" max="3" width="3.109375" customWidth="1"/>
-    <col min="4" max="4" width="26.77734375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="3.21875" customWidth="1"/>
-    <col min="6" max="6" width="67.109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="109.5546875" customWidth="1"/>
-    <col min="8" max="8" width="27.21875" customWidth="1"/>
+    <col min="1" max="1" width="8.33203125" customWidth="1"/>
+    <col min="2" max="2" width="3" customWidth="1"/>
+    <col min="3" max="3" width="2.5546875" customWidth="1"/>
+    <col min="4" max="4" width="24.21875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="2.109375" customWidth="1"/>
+    <col min="6" max="6" width="65.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="33.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1601,7 +1564,7 @@
         <v>12</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>307</v>
+        <v>284</v>
       </c>
       <c r="H2" t="s">
         <v>13</v>
@@ -1627,7 +1590,7 @@
         <v>15</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>281</v>
+        <v>252</v>
       </c>
       <c r="H3" t="s">
         <v>16</v>
@@ -1653,7 +1616,7 @@
         <v>19</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="H4" t="s">
         <v>20</v>
@@ -1679,7 +1642,7 @@
         <v>23</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>294</v>
+        <v>256</v>
       </c>
       <c r="H5" t="s">
         <v>24</v>
@@ -1705,7 +1668,7 @@
         <v>26</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>279</v>
+        <v>253</v>
       </c>
       <c r="H6" t="s">
         <v>27</v>
@@ -1731,7 +1694,7 @@
         <v>19</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="H7" t="s">
         <v>20</v>
@@ -1757,7 +1720,7 @@
         <v>30</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="H8" t="s">
         <v>31</v>
@@ -1783,7 +1746,7 @@
         <v>26</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>279</v>
+        <v>253</v>
       </c>
       <c r="H9" t="s">
         <v>27</v>
@@ -1809,7 +1772,7 @@
         <v>33</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="H10" t="s">
         <v>34</v>
@@ -1835,7 +1798,7 @@
         <v>30</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="H11" t="s">
         <v>31</v>
@@ -1861,7 +1824,7 @@
         <v>15</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>281</v>
+        <v>252</v>
       </c>
       <c r="H12" t="s">
         <v>16</v>
@@ -1887,7 +1850,7 @@
         <v>37</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="H13" t="s">
         <v>38</v>
@@ -1913,7 +1876,7 @@
         <v>12</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>307</v>
+        <v>284</v>
       </c>
       <c r="H14" t="s">
         <v>13</v>
@@ -1939,7 +1902,7 @@
         <v>15</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>281</v>
+        <v>252</v>
       </c>
       <c r="H15" t="s">
         <v>16</v>
@@ -1965,7 +1928,7 @@
         <v>37</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="H16" t="s">
         <v>38</v>
@@ -1991,7 +1954,7 @@
         <v>23</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>294</v>
+        <v>256</v>
       </c>
       <c r="H17" t="s">
         <v>24</v>
@@ -2017,7 +1980,7 @@
         <v>26</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>279</v>
+        <v>253</v>
       </c>
       <c r="H18" t="s">
         <v>27</v>
@@ -2043,7 +2006,7 @@
         <v>37</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="H19" t="s">
         <v>38</v>
@@ -2069,7 +2032,7 @@
         <v>44</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>305</v>
+        <v>288</v>
       </c>
       <c r="H20" t="s">
         <v>45</v>
@@ -2095,7 +2058,7 @@
         <v>47</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H21" t="s">
         <v>48</v>
@@ -2121,7 +2084,7 @@
         <v>51</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>291</v>
+        <v>254</v>
       </c>
       <c r="H22" t="s">
         <v>52</v>
@@ -2147,7 +2110,7 @@
         <v>54</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>299</v>
+        <v>258</v>
       </c>
       <c r="H23" t="s">
         <v>55</v>
@@ -2173,7 +2136,7 @@
         <v>58</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="H24" t="s">
         <v>59</v>
@@ -2199,7 +2162,7 @@
         <v>47</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H25" t="s">
         <v>48</v>
@@ -2215,20 +2178,20 @@
       <c r="C26">
         <v>1</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>252</v>
+      <c r="D26" t="s">
+        <v>61</v>
       </c>
       <c r="E26" t="s">
         <v>18</v>
       </c>
       <c r="F26" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>292</v>
+        <v>278</v>
       </c>
       <c r="H26" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -2251,7 +2214,7 @@
         <v>54</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>299</v>
+        <v>258</v>
       </c>
       <c r="H27" t="s">
         <v>55</v>
@@ -2262,7 +2225,7 @@
         <v>41</v>
       </c>
       <c r="B28" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -2277,7 +2240,7 @@
         <v>44</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>305</v>
+        <v>288</v>
       </c>
       <c r="H28" t="s">
         <v>45</v>
@@ -2288,7 +2251,7 @@
         <v>41</v>
       </c>
       <c r="B29" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C29">
         <v>2</v>
@@ -2303,7 +2266,7 @@
         <v>54</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>299</v>
+        <v>258</v>
       </c>
       <c r="H29" t="s">
         <v>55</v>
@@ -2314,7 +2277,7 @@
         <v>41</v>
       </c>
       <c r="B30" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -2329,7 +2292,7 @@
         <v>51</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>291</v>
+        <v>254</v>
       </c>
       <c r="H30" t="s">
         <v>52</v>
@@ -2340,7 +2303,7 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C31">
         <v>2</v>
@@ -2355,7 +2318,7 @@
         <v>47</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H31" t="s">
         <v>48</v>
@@ -2363,2456 +2326,2436 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B32" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C32">
         <v>1</v>
       </c>
       <c r="D32" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E32" t="s">
         <v>11</v>
       </c>
       <c r="F32" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="H32" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B33" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C33">
         <v>2</v>
       </c>
       <c r="D33" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E33" t="s">
         <v>11</v>
       </c>
       <c r="F33" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>304</v>
+        <v>285</v>
       </c>
       <c r="H33" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B34" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C34">
         <v>3</v>
       </c>
       <c r="D34" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E34" t="s">
         <v>11</v>
       </c>
       <c r="F34" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H34" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C35">
         <v>1</v>
       </c>
       <c r="D35" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E35" t="s">
         <v>11</v>
       </c>
       <c r="F35" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:8">
       <c r="A36" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B36" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C36">
         <v>2</v>
       </c>
       <c r="D36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E36" t="s">
         <v>11</v>
       </c>
       <c r="F36" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="H36" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" spans="1:8">
       <c r="A37" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C37">
         <v>3</v>
       </c>
       <c r="D37" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E37" t="s">
         <v>11</v>
       </c>
       <c r="F37" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="H37" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:8">
       <c r="A38" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B38" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C38">
         <v>1</v>
       </c>
       <c r="D38" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E38" t="s">
         <v>11</v>
       </c>
       <c r="F38" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="H38" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B39" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C39">
         <v>2</v>
       </c>
       <c r="D39" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E39" t="s">
         <v>11</v>
       </c>
       <c r="F39" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="H39" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B40" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C40">
         <v>3</v>
       </c>
       <c r="D40" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E40" t="s">
         <v>18</v>
       </c>
       <c r="F40" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
       <c r="H40" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="41" spans="1:8">
       <c r="A41" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B41" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E41" t="s">
         <v>11</v>
       </c>
       <c r="F41" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H41" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="42" spans="1:8">
       <c r="A42" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B42" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C42">
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E42" t="s">
         <v>11</v>
       </c>
       <c r="F42" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="H42" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" spans="1:8">
       <c r="A43" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B43" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C43">
         <v>3</v>
       </c>
       <c r="D43" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E43" t="s">
         <v>18</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>288</v>
+        <v>255</v>
       </c>
       <c r="H43" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B44" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C44">
         <v>1</v>
       </c>
       <c r="D44" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E44" t="s">
         <v>11</v>
       </c>
       <c r="F44" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>304</v>
+        <v>285</v>
       </c>
       <c r="H44" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="45" spans="1:8">
       <c r="A45" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B45" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C45">
         <v>2</v>
       </c>
       <c r="D45" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E45" t="s">
         <v>11</v>
       </c>
       <c r="F45" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H45" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="46" spans="1:8">
       <c r="A46" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B46" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C46">
         <v>3</v>
       </c>
       <c r="D46" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E46" t="s">
         <v>18</v>
       </c>
       <c r="F46" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="H46" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="47" spans="1:8">
       <c r="A47" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B47" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C47">
         <v>1</v>
       </c>
       <c r="D47" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E47" t="s">
         <v>11</v>
       </c>
       <c r="F47" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="H47" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="48" spans="1:8">
       <c r="A48" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B48" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C48">
         <v>2</v>
       </c>
       <c r="D48" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E48" t="s">
         <v>11</v>
       </c>
       <c r="F48" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H48" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="49" spans="1:8">
       <c r="A49" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B49" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C49">
         <v>3</v>
       </c>
       <c r="D49" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E49" t="s">
         <v>11</v>
       </c>
       <c r="F49" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="H49" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="50" spans="1:8">
       <c r="A50" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B50" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C50">
         <v>1</v>
       </c>
       <c r="D50" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E50" t="s">
         <v>18</v>
       </c>
       <c r="F50" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>306</v>
+        <v>287</v>
       </c>
       <c r="H50" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="51" spans="1:8">
       <c r="A51" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B51" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C51">
         <v>2</v>
       </c>
       <c r="D51" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E51" t="s">
         <v>18</v>
       </c>
       <c r="F51" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="H51" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="52" spans="1:8">
       <c r="A52" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B52" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C52">
         <v>1</v>
       </c>
       <c r="D52" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E52" t="s">
         <v>18</v>
       </c>
       <c r="F52" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="H52" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="53" spans="1:8">
       <c r="A53" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B53" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C53">
         <v>2</v>
       </c>
       <c r="D53" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E53" t="s">
         <v>18</v>
       </c>
       <c r="F53" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="H53" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="54" spans="1:8">
       <c r="A54" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B54" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C54">
         <v>1</v>
       </c>
       <c r="D54" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E54" t="s">
         <v>18</v>
       </c>
       <c r="F54" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>300</v>
+        <v>286</v>
       </c>
       <c r="H54" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="55" spans="1:8">
       <c r="A55" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B55" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C55">
         <v>2</v>
       </c>
       <c r="D55" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E55" t="s">
         <v>18</v>
       </c>
       <c r="F55" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="H55" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="56" spans="1:8">
       <c r="A56" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B56" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C56">
         <v>1</v>
       </c>
       <c r="D56" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E56" t="s">
         <v>18</v>
       </c>
       <c r="F56" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>306</v>
+        <v>287</v>
       </c>
       <c r="H56" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="57" spans="1:8">
       <c r="A57" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B57" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C57">
         <v>2</v>
       </c>
       <c r="D57" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E57" t="s">
         <v>18</v>
       </c>
       <c r="F57" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="H57" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="58" spans="1:8">
       <c r="A58" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B58" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C58">
         <v>1</v>
       </c>
       <c r="D58" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E58" t="s">
         <v>18</v>
       </c>
       <c r="F58" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="H58" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="59" spans="1:8">
       <c r="A59" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B59" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C59">
         <v>2</v>
       </c>
       <c r="D59" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E59" t="s">
         <v>18</v>
       </c>
       <c r="F59" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="H59" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="60" spans="1:8">
       <c r="A60" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B60" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C60">
         <v>1</v>
       </c>
       <c r="D60" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E60" t="s">
         <v>18</v>
       </c>
       <c r="F60" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>300</v>
+        <v>286</v>
       </c>
       <c r="H60" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="61" spans="1:8">
       <c r="A61" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B61" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C61">
         <v>2</v>
       </c>
       <c r="D61" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E61" t="s">
         <v>18</v>
       </c>
       <c r="F61" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="H61" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="62" spans="1:8">
       <c r="A62" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B62" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C62">
         <v>1</v>
       </c>
       <c r="D62" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E62" t="s">
         <v>18</v>
       </c>
       <c r="F62" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="H62" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="63" spans="1:8">
       <c r="A63" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B63" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C63">
         <v>2</v>
       </c>
       <c r="D63" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E63" t="s">
         <v>18</v>
       </c>
       <c r="F63" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="H63" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="64" spans="1:8">
       <c r="A64" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B64" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C64">
         <v>1</v>
       </c>
       <c r="D64" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E64" t="s">
         <v>18</v>
       </c>
       <c r="F64" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="H64" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="65" spans="1:8">
       <c r="A65" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B65" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C65">
         <v>2</v>
       </c>
       <c r="D65" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E65" t="s">
         <v>11</v>
       </c>
       <c r="F65" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>298</v>
+        <v>257</v>
       </c>
       <c r="H65" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="66" spans="1:8">
       <c r="A66" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B66" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C66">
         <v>1</v>
       </c>
-      <c r="D66" s="6" t="s">
-        <v>140</v>
+      <c r="D66" t="s">
+        <v>141</v>
       </c>
       <c r="E66" t="s">
         <v>11</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>310</v>
+        <v>268</v>
       </c>
       <c r="H66" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="67" spans="1:8">
       <c r="A67" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B67" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C67">
         <v>2</v>
       </c>
-      <c r="D67" s="6" t="s">
-        <v>143</v>
+      <c r="D67" t="s">
+        <v>144</v>
       </c>
       <c r="E67" t="s">
         <v>18</v>
       </c>
       <c r="F67" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="H67" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="68" spans="1:8">
       <c r="A68" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B68" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C68">
         <v>1</v>
       </c>
       <c r="D68" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E68" t="s">
         <v>18</v>
       </c>
       <c r="F68" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>309</v>
+        <v>273</v>
       </c>
       <c r="H68" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="69" spans="1:8">
       <c r="A69" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B69" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C69">
         <v>2</v>
       </c>
       <c r="D69" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E69" t="s">
         <v>11</v>
       </c>
       <c r="F69" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="H69" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="70" spans="1:8">
       <c r="A70" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B70" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C70">
         <v>1</v>
       </c>
       <c r="D70" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E70" t="s">
         <v>18</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="H70" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="71" spans="1:8">
       <c r="A71" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B71" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C71">
         <v>2</v>
       </c>
       <c r="D71" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E71" t="s">
         <v>18</v>
       </c>
       <c r="F71" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="H71" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="72" spans="1:8">
       <c r="A72" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B72" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C72">
         <v>1</v>
       </c>
       <c r="D72" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E72" t="s">
         <v>18</v>
       </c>
       <c r="F72" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="H72" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="73" spans="1:8">
       <c r="A73" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B73" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C73">
         <v>2</v>
       </c>
       <c r="D73" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E73" t="s">
         <v>11</v>
       </c>
       <c r="F73" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>297</v>
+        <v>282</v>
       </c>
       <c r="H73" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="74" spans="1:8">
       <c r="A74" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B74" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C74">
         <v>1</v>
       </c>
       <c r="D74" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E74" t="s">
         <v>11</v>
       </c>
       <c r="F74" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>275</v>
+        <v>298</v>
       </c>
       <c r="H74" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="75" spans="1:8">
       <c r="A75" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B75" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C75">
         <v>2</v>
       </c>
       <c r="D75" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E75" t="s">
         <v>18</v>
       </c>
       <c r="F75" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>272</v>
+        <v>303</v>
       </c>
       <c r="H75" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="76" spans="1:8">
       <c r="A76" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B76" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C76">
         <v>3</v>
       </c>
       <c r="D76" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E76" t="s">
         <v>18</v>
       </c>
       <c r="F76" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>283</v>
+        <v>300</v>
       </c>
       <c r="H76" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="77" spans="1:8">
       <c r="A77" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B77" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C77">
         <v>4</v>
       </c>
       <c r="D77" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E77" t="s">
         <v>18</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>282</v>
+        <v>297</v>
       </c>
       <c r="H77" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="78" spans="1:8">
       <c r="A78" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B78" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C78">
         <v>5</v>
       </c>
       <c r="D78" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E78" t="s">
         <v>18</v>
       </c>
       <c r="F78" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>257</v>
+        <v>309</v>
       </c>
       <c r="H78" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="79" spans="1:8">
       <c r="A79" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B79" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C79">
         <v>6</v>
       </c>
       <c r="D79" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E79" t="s">
         <v>11</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
       <c r="H79" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="80" spans="1:8">
       <c r="A80" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B80" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C80">
         <v>1</v>
       </c>
       <c r="D80" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E80" t="s">
         <v>11</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
       <c r="H80" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="81" spans="1:8">
       <c r="A81" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B81" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C81">
         <v>2</v>
       </c>
       <c r="D81" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E81" t="s">
         <v>18</v>
       </c>
       <c r="F81" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>272</v>
+        <v>303</v>
       </c>
       <c r="H81" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="82" spans="1:8">
       <c r="A82" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B82" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C82">
         <v>3</v>
       </c>
       <c r="D82" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E82" t="s">
         <v>18</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G82" s="3" t="s">
-        <v>276</v>
+        <v>301</v>
       </c>
       <c r="H82" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="83" spans="1:8">
       <c r="A83" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B83" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C83">
         <v>4</v>
       </c>
       <c r="D83" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E83" t="s">
         <v>18</v>
       </c>
       <c r="F83" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>262</v>
+        <v>308</v>
       </c>
       <c r="H83" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="84" spans="1:8">
       <c r="A84" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B84" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C84">
         <v>5</v>
       </c>
       <c r="D84" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E84" t="s">
         <v>18</v>
       </c>
       <c r="F84" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>283</v>
+        <v>300</v>
       </c>
       <c r="H84" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="85" spans="1:8">
       <c r="A85" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B85" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C85">
         <v>6</v>
       </c>
-      <c r="D85" s="5" t="s">
-        <v>253</v>
+      <c r="D85" t="s">
+        <v>187</v>
       </c>
       <c r="E85" t="s">
         <v>11</v>
       </c>
       <c r="F85" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>265</v>
+        <v>306</v>
       </c>
       <c r="H85" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="86" spans="1:8">
       <c r="A86" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B86" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C86">
         <v>1</v>
       </c>
       <c r="D86" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E86" t="s">
         <v>11</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G86" s="3" t="s">
-        <v>285</v>
+        <v>295</v>
       </c>
       <c r="H86" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="87" spans="1:8">
       <c r="A87" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B87" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C87">
         <v>2</v>
       </c>
       <c r="D87" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E87" t="s">
         <v>11</v>
       </c>
       <c r="F87" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G87" s="3" t="s">
         <v>261</v>
       </c>
       <c r="H87" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="88" spans="1:8">
       <c r="A88" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B88" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C88">
         <v>3</v>
       </c>
       <c r="D88" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E88" t="s">
         <v>18</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="H88" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="89" spans="1:8">
       <c r="A89" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B89" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C89">
         <v>4</v>
       </c>
       <c r="D89" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E89" t="s">
         <v>18</v>
       </c>
       <c r="F89" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>257</v>
+        <v>309</v>
       </c>
       <c r="H89" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="90" spans="1:8">
       <c r="A90" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B90" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C90">
         <v>5</v>
       </c>
       <c r="D90" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E90" t="s">
         <v>18</v>
       </c>
       <c r="F90" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>283</v>
+        <v>300</v>
       </c>
       <c r="H90" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="91" spans="1:8">
       <c r="A91" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B91" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C91">
         <v>6</v>
       </c>
       <c r="D91" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E91" t="s">
         <v>18</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>276</v>
+        <v>301</v>
       </c>
       <c r="H91" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="92" spans="1:8">
       <c r="A92" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B92" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C92">
         <v>1</v>
       </c>
       <c r="D92" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E92" t="s">
         <v>11</v>
       </c>
       <c r="F92" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>303</v>
+        <v>259</v>
       </c>
       <c r="H92" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="93" spans="1:8">
       <c r="A93" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B93" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C93">
         <v>2</v>
       </c>
       <c r="D93" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E93" t="s">
         <v>11</v>
       </c>
       <c r="F93" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>275</v>
+        <v>298</v>
       </c>
       <c r="H93" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="94" spans="1:8">
       <c r="A94" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B94" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C94">
         <v>3</v>
       </c>
       <c r="D94" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E94" t="s">
         <v>18</v>
       </c>
       <c r="F94" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G94" s="3" t="s">
         <v>261</v>
       </c>
       <c r="H94" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="95" spans="1:8">
       <c r="A95" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B95" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C95">
         <v>4</v>
       </c>
       <c r="D95" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E95" t="s">
         <v>18</v>
       </c>
       <c r="F95" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G95" s="3" t="s">
-        <v>257</v>
+        <v>309</v>
       </c>
       <c r="H95" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="96" spans="1:8">
       <c r="A96" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B96" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C96">
         <v>5</v>
       </c>
       <c r="D96" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E96" t="s">
         <v>18</v>
       </c>
       <c r="F96" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G96" s="3" t="s">
-        <v>283</v>
+        <v>300</v>
       </c>
       <c r="H96" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="97" spans="1:8">
       <c r="A97" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B97" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C97">
         <v>6</v>
       </c>
       <c r="D97" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E97" t="s">
         <v>18</v>
       </c>
       <c r="F97" s="1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G97" s="3" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="H97" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="98" spans="1:8">
       <c r="A98" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B98" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C98">
         <v>1</v>
       </c>
       <c r="D98" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E98" t="s">
         <v>11</v>
       </c>
       <c r="F98" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G98" s="3" t="s">
-        <v>303</v>
+        <v>259</v>
       </c>
       <c r="H98" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="99" spans="1:8">
       <c r="A99" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B99" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C99">
         <v>2</v>
       </c>
       <c r="D99" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E99" t="s">
         <v>18</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G99" s="3" t="s">
-        <v>276</v>
+        <v>301</v>
       </c>
       <c r="H99" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="100" spans="1:8">
       <c r="A100" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B100" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C100">
         <v>3</v>
       </c>
       <c r="D100" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E100" t="s">
         <v>18</v>
       </c>
       <c r="F100" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G100" s="3" t="s">
-        <v>272</v>
+        <v>303</v>
       </c>
       <c r="H100" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="101" spans="1:8">
       <c r="A101" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B101" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C101">
         <v>4</v>
       </c>
       <c r="D101" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E101" t="s">
         <v>18</v>
       </c>
       <c r="F101" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G101" s="3" t="s">
-        <v>257</v>
+        <v>309</v>
       </c>
       <c r="H101" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="102" spans="1:8">
       <c r="A102" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B102" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C102">
         <v>5</v>
       </c>
       <c r="D102" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E102" t="s">
         <v>18</v>
       </c>
       <c r="F102" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G102" s="3" t="s">
-        <v>283</v>
+        <v>300</v>
       </c>
       <c r="H102" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="103" spans="1:8">
       <c r="A103" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B103" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C103">
         <v>6</v>
       </c>
       <c r="D103" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E103" t="s">
         <v>18</v>
       </c>
       <c r="F103" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G103" s="3" t="s">
-        <v>262</v>
+        <v>308</v>
       </c>
       <c r="H103" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="104" spans="1:8">
       <c r="A104" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B104" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C104">
         <v>1</v>
       </c>
       <c r="D104" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E104" t="s">
         <v>11</v>
       </c>
       <c r="F104" s="1" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="G104" s="3" t="s">
-        <v>303</v>
+        <v>259</v>
       </c>
       <c r="H104" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="105" spans="1:8">
       <c r="A105" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B105" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C105">
         <v>2</v>
       </c>
       <c r="D105" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E105" t="s">
         <v>11</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G105" s="3" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
       <c r="H105" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="106" spans="1:8">
       <c r="A106" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B106" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C106">
         <v>3</v>
       </c>
       <c r="D106" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E106" t="s">
         <v>18</v>
       </c>
       <c r="F106" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G106" s="3" t="s">
         <v>261</v>
       </c>
       <c r="H106" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="107" spans="1:8">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B107" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C107">
         <v>4</v>
       </c>
       <c r="D107" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E107" t="s">
         <v>18</v>
       </c>
       <c r="F107" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G107" s="3" t="s">
-        <v>257</v>
+        <v>309</v>
       </c>
       <c r="H107" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="108" spans="1:8">
       <c r="A108" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B108" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C108">
         <v>5</v>
       </c>
       <c r="D108" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E108" t="s">
         <v>18</v>
       </c>
       <c r="F108" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G108" s="3" t="s">
-        <v>283</v>
+        <v>300</v>
       </c>
       <c r="H108" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="109" spans="1:8">
       <c r="A109" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B109" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C109">
         <v>6</v>
       </c>
       <c r="D109" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E109" t="s">
         <v>18</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G109" s="3" t="s">
-        <v>282</v>
+        <v>297</v>
       </c>
       <c r="H109" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="110" spans="1:8">
       <c r="A110" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B110" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C110">
         <v>1</v>
       </c>
       <c r="D110" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E110" t="s">
         <v>18</v>
       </c>
       <c r="F110" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="G110" s="3" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="H110" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="111" spans="1:8">
       <c r="A111" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B111" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C111">
         <v>2</v>
       </c>
       <c r="D111" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E111" t="s">
         <v>18</v>
       </c>
       <c r="F111" s="1" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G111" s="3" t="s">
-        <v>274</v>
+        <v>299</v>
       </c>
       <c r="H111" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="112" spans="1:8">
       <c r="A112" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B112" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C112">
         <v>1</v>
       </c>
       <c r="D112" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="E112" t="s">
         <v>18</v>
       </c>
       <c r="F112" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="G112" s="3" t="s">
-        <v>267</v>
+        <v>305</v>
       </c>
       <c r="H112" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="113" spans="1:8">
       <c r="A113" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B113" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C113">
         <v>2</v>
       </c>
       <c r="D113" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E113" t="s">
         <v>18</v>
       </c>
       <c r="F113" s="1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G113" s="3" t="s">
-        <v>263</v>
+        <v>307</v>
       </c>
       <c r="H113" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="114" spans="1:8">
       <c r="A114" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B114" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C114">
         <v>1</v>
       </c>
       <c r="D114" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="E114" t="s">
         <v>18</v>
       </c>
       <c r="F114" s="1" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G114" s="3" t="s">
-        <v>311</v>
+        <v>291</v>
       </c>
       <c r="H114" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="115" spans="1:8">
       <c r="A115" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B115" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C115">
         <v>2</v>
       </c>
       <c r="D115" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E115" t="s">
         <v>18</v>
       </c>
       <c r="G115" s="3" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="H115" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="116" spans="1:8">
       <c r="A116" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B116" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C116">
         <v>1</v>
       </c>
       <c r="D116" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E116" t="s">
         <v>18</v>
       </c>
       <c r="F116" s="1" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="G116" s="3" t="s">
-        <v>269</v>
+        <v>304</v>
       </c>
       <c r="H116" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="117" spans="1:8">
       <c r="A117" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B117" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C117">
         <v>2</v>
       </c>
       <c r="D117" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E117" t="s">
         <v>18</v>
       </c>
       <c r="F117" s="1" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="G117" s="3" t="s">
-        <v>308</v>
+        <v>260</v>
       </c>
       <c r="H117" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="118" spans="1:8">
       <c r="A118" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B118" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C118">
         <v>1</v>
       </c>
       <c r="D118" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E118" t="s">
         <v>18</v>
       </c>
       <c r="F118" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G118" s="3" t="s">
-        <v>274</v>
+        <v>299</v>
       </c>
       <c r="H118" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="119" spans="1:8">
       <c r="A119" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B119" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C119">
         <v>2</v>
       </c>
       <c r="D119" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E119" t="s">
         <v>18</v>
       </c>
       <c r="F119" s="1" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G119" s="3" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="H119" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="120" spans="1:8">
       <c r="A120" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B120" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C120">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D120" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E120" t="s">
         <v>18</v>
       </c>
+      <c r="F120" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="G120" s="3" t="s">
+        <v>294</v>
+      </c>
       <c r="H120" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="121" spans="1:8">
-      <c r="A121" t="s">
-        <v>211</v>
-      </c>
-      <c r="B121" t="s">
-        <v>246</v>
-      </c>
-      <c r="C121">
-        <v>2</v>
-      </c>
-      <c r="D121" t="s">
-        <v>249</v>
-      </c>
-      <c r="E121" t="s">
-        <v>18</v>
-      </c>
-      <c r="F121" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="G121" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="H121" t="s">
         <v>251</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G10" r:id="rId1" xr:uid="{19105C44-55F9-4FCB-9097-095014F9DA3E}"/>
-    <hyperlink ref="G39" r:id="rId2" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631432/moveon/Final_Images/T-Bar Rows.webp" xr:uid="{3357DAF4-CEF1-4A2D-A618-5038B3D80DA2}"/>
-    <hyperlink ref="G40" r:id="rId3" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Straight Arm Pulldowns.webp" xr:uid="{DF101A74-11D1-4D48-A55F-70CD6E36B882}"/>
-    <hyperlink ref="G59" r:id="rId4" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631430/moveon/Final_Images/Spider Curls.webp" xr:uid="{3DB28FB9-989B-4FAB-84D8-7325E7168A51}"/>
-    <hyperlink ref="G38" r:id="rId5" xr:uid="{DDB839C0-F533-4CD6-82BA-9C7BE1D74535}"/>
-    <hyperlink ref="G42" r:id="rId6" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631427/moveon/Final_Images/Seated Rows Close-Grip.webp" xr:uid="{D84C3733-7D70-4CFF-9839-4F853A55D44D}"/>
-    <hyperlink ref="G94" r:id="rId7" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631426/moveon/Final_Images/Seated Leg Curl.webp" xr:uid="{64D59DE8-0E5D-4EA3-9A52-262F81DFB538}"/>
-    <hyperlink ref="G113" r:id="rId8" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631422/moveon/Final_Images/Russian Twists.webp" xr:uid="{97DD529F-65CB-4D95-9D52-23D3CE53F56E}"/>
-    <hyperlink ref="G63" r:id="rId9" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Rope Pushdowns.webp" xr:uid="{C5953424-AA18-47AE-A2F7-B9AFD2114352}"/>
-    <hyperlink ref="G85" r:id="rId10" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Romani Deadleft.webp" xr:uid="{AECD93F6-DA69-4D96-A009-6B5233BF04D4}"/>
-    <hyperlink ref="G53" r:id="rId11" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631420/moveon/Final_Images/Preacher Curls.webp" xr:uid="{51671F7D-7442-420A-815E-A27B5AAB5C02}"/>
-    <hyperlink ref="G112" r:id="rId12" xr:uid="{02EB4EB2-1057-4F42-B6C0-540B51CC23C0}"/>
-    <hyperlink ref="G13" r:id="rId13" xr:uid="{055FE933-E563-46DE-991F-CED9B287397A}"/>
-    <hyperlink ref="G116" r:id="rId14" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631418/moveon/Final_Images/Mountain Climbers.webp" xr:uid="{7F58DA86-9CE7-4B97-B895-8A5A94C4A5C0}"/>
-    <hyperlink ref="G24" r:id="rId15" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631417/moveon/Final_Images/Machine Shoulder Press.webp" xr:uid="{177FF476-981A-4802-8E74-D96A2EAB1E04}"/>
-    <hyperlink ref="G8" r:id="rId16" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631416/moveon/Final_Images/Machine Bench Press.webp" xr:uid="{23AE3FBD-B6FC-4F81-827E-10D6BFA8C47E}"/>
-    <hyperlink ref="G100" r:id="rId17" xr:uid="{BEC30C2A-A013-424A-B5BD-8E72787A84AD}"/>
-    <hyperlink ref="G105" r:id="rId18" xr:uid="{9E7AAEB7-6D2F-4DB1-B3A8-2A2F414BF2C1}"/>
-    <hyperlink ref="G37" r:id="rId19" xr:uid="{E4491B30-BE87-4A2D-A73F-E488D0FB7EBA}"/>
-    <hyperlink ref="G111" r:id="rId20" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631413/moveon/Final_Images/Leg Raises.webp" xr:uid="{406C5C5C-69CE-4CEA-978E-3B94865E52B4}"/>
-    <hyperlink ref="G74" r:id="rId21" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631413/moveon/Final_Images/Leg Press.webp" xr:uid="{724AC210-EEB5-46CF-B310-BEE8B9350490}"/>
-    <hyperlink ref="G82" r:id="rId22" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631412/moveon/Final_Images/Leg Extensions.webp" xr:uid="{66EBA1DB-799F-406C-84D5-6B3500581E18}"/>
-    <hyperlink ref="G21" r:id="rId23" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631411/moveon/Final_Images/Lateral Raises.webp" xr:uid="{F380D370-7BE9-4599-9D0D-4F0FC499A8A1}"/>
-    <hyperlink ref="G34" r:id="rId24" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631410/moveon/Final_Images/Lat Pulldowns.webp" xr:uid="{A77C1117-51C9-4944-981B-11FD17350623}"/>
-    <hyperlink ref="G35" r:id="rId25" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631410/moveon/Final_Images/Lat Pulldowns.webp" xr:uid="{6AEF8481-2161-4A9B-9C5A-86B3510FEBDB}"/>
-    <hyperlink ref="G6" r:id="rId26" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline Dumbbell Press.webp" xr:uid="{3DF49E4A-B9A6-4221-A806-59986067EFCA}"/>
-    <hyperlink ref="G57" r:id="rId27" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline Dumbbell Curls.webp" xr:uid="{9A524B8B-D0D9-4430-AE72-E01D0B2974C7}"/>
-    <hyperlink ref="G3" r:id="rId28" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631408/moveon/Final_Images/Incline Barbell Press.webp" xr:uid="{1B0795C6-92C3-4C25-9553-BABC3A4C5D29}"/>
-    <hyperlink ref="G109" r:id="rId29" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Thrust.webp" xr:uid="{3E2C1B7D-99E1-44DE-8499-36926F260455}"/>
-    <hyperlink ref="G102" r:id="rId30" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Adductor Machine.webp" xr:uid="{BF0D7FDE-0AB4-423D-BCA9-6293F7983A86}"/>
-    <hyperlink ref="G108" r:id="rId31" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Adductor Machine.webp" xr:uid="{6F3A60A1-1B14-481E-A73E-9C5436E7310D}"/>
-    <hyperlink ref="G115" r:id="rId32" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631406/moveon/Final_Images/Hanging Knee Raises.webp" xr:uid="{E12AABA4-A146-4865-A680-15E6F9EA667B}"/>
-    <hyperlink ref="G86" r:id="rId33" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631405/moveon/Final_Images/Hack Squats.webp" xr:uid="{152783E0-4E0D-4990-AC04-8971CEB21A9F}"/>
-    <hyperlink ref="G97" r:id="rId34" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631405/moveon/Final_Images/Glute Bridges.webp" xr:uid="{9B314E4A-043A-474E-A39C-2CC5E4C916F4}"/>
-    <hyperlink ref="G121" r:id="rId35" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631403/moveon/Final_Images/Flutter Kicks.webp" xr:uid="{A6A2F371-2ABE-4357-AB9B-1696E3F5E757}"/>
-    <hyperlink ref="G43" r:id="rId36" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631402/moveon/Final_Images/Face Pulls.webp" xr:uid="{22654AD9-6C0B-4113-9628-8246E7345A20}"/>
-    <hyperlink ref="G62" r:id="rId37" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631402/moveon/Final_Images/Dumbbell Tricep Kickback.webp" xr:uid="{00C36918-7540-4107-A53A-5A837130F0D4}"/>
-    <hyperlink ref="G36" r:id="rId38" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631401/moveon/Final_Images/Dumbbell Rows.webp" xr:uid="{0C753DF4-09A9-4B03-920E-849D848F462A}"/>
-    <hyperlink ref="G22" r:id="rId39" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631400/moveon/Final_Images/Dumbbell Overhead Press.webp" xr:uid="{316F5ACB-5893-4A79-9F87-FA14CA93FE30}"/>
-    <hyperlink ref="G26" r:id="rId40" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631399/moveon/Final_Images/Dumbbell Front Raises.webp" xr:uid="{044B8EE7-F039-4487-8023-834AD7C1246D}"/>
-    <hyperlink ref="G52" r:id="rId41" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631398/moveon/Final_Images/Dumbbell Curls.webp" xr:uid="{5ADF9132-C856-4C83-978E-67D48D4AC5A2}"/>
-    <hyperlink ref="G5" r:id="rId42" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631398/moveon/Final_Images/Dumbbell Bench Press.webp" xr:uid="{221C1554-894C-42DD-BA7C-24A1D253C005}"/>
-    <hyperlink ref="G51" r:id="rId43" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631396/moveon/Final_Images/Concentration Curls.webp" xr:uid="{D68DE0C3-B0BF-4332-9EC9-45D32B77AA1C}"/>
-    <hyperlink ref="G110" r:id="rId44" xr:uid="{4E8B250D-0E32-4383-BADC-3429C7B0B4EC}"/>
-    <hyperlink ref="G73" r:id="rId45" xr:uid="{B3ACAA6A-7137-4CA7-A2F5-46205CE6CFC8}"/>
-    <hyperlink ref="G65" r:id="rId46" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631395/moveon/Final_Images/Close-Grip Bench Press.webp" xr:uid="{D4FA6B07-0990-49AA-9601-9806EE2869FF}"/>
-    <hyperlink ref="G27" r:id="rId47" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631394/moveon/Final_Images/Cable Lateral Raises.webp" xr:uid="{A6B189E5-A81D-495F-B571-69B59D51DCAB}"/>
-    <hyperlink ref="G54" r:id="rId48" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631393/moveon/Final_Images/Cable Curls.webp" xr:uid="{E4CABCAC-C0DC-491B-A1D6-135EA36263F8}"/>
-    <hyperlink ref="G4" r:id="rId49" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631392/moveon/Final_Images/Cable Crossovers High to Low.webp" xr:uid="{50D44733-022A-41E3-A737-73DD9F3B7F0C}"/>
-    <hyperlink ref="G119" r:id="rId50" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631392/moveon/Final_Images/Bicycle Crunches.webp" xr:uid="{C2904B5E-3C9D-4CEC-8B7B-E2325905471A}"/>
-    <hyperlink ref="G92" r:id="rId51" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell Squats.webp" xr:uid="{BFF8B31F-67C3-460C-80A5-AAEF2F0BA911}"/>
-    <hyperlink ref="G33" r:id="rId52" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell Rows.webp" xr:uid="{FCC625F9-46E2-4399-A404-AED539CB8700}"/>
-    <hyperlink ref="G20" r:id="rId53" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631390/moveon/Final_Images/Barbell Overhead Press.webp" xr:uid="{54BC23DE-406D-4B96-87F3-D1DE83BDB059}"/>
-    <hyperlink ref="G50" r:id="rId54" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631389/moveon/Final_Images/Barbell Curls.webp" xr:uid="{1C564B66-22F8-4374-8D4F-AE01309211B1}"/>
-    <hyperlink ref="G2" r:id="rId55" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631388/moveon/Final_Images/Barbell Bench Press.webp" xr:uid="{5982C014-79E2-4A41-BFCD-49EC560F3613}"/>
-    <hyperlink ref="G117" r:id="rId56" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631387/moveon/Final_Images/Ab Wheel Rollouts.webp" xr:uid="{6255A00E-FA00-4393-AFD8-3CBF85A1DB7D}"/>
-    <hyperlink ref="G7" r:id="rId57" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631392/moveon/Final_Images/Cable Crossovers High to Low.webp" xr:uid="{88C66FAC-C3CE-4EEB-8E30-90D4CA3E72DF}"/>
-    <hyperlink ref="G14" r:id="rId58" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631388/moveon/Final_Images/Barbell Bench Press.webp" xr:uid="{CCC14FC3-05A0-4FE3-B7A1-6154F59D55D6}"/>
-    <hyperlink ref="G12" r:id="rId59" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631408/moveon/Final_Images/Incline Barbell Press.webp" xr:uid="{33B87BF1-6B67-4CA3-8197-A9A776E9086F}"/>
-    <hyperlink ref="G15" r:id="rId60" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631408/moveon/Final_Images/Incline Barbell Press.webp" xr:uid="{EE816864-75C5-4CA4-A517-639316DECAF1}"/>
-    <hyperlink ref="G17" r:id="rId61" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631398/moveon/Final_Images/Dumbbell Bench Press.webp" xr:uid="{C424288C-7FDF-488D-829E-1465057B85A4}"/>
-    <hyperlink ref="G11" r:id="rId62" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631416/moveon/Final_Images/Machine Bench Press.webp" xr:uid="{94A8A25E-E17F-4126-A006-DC5B52F82C4B}"/>
-    <hyperlink ref="G9" r:id="rId63" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline Dumbbell Press.webp" xr:uid="{F02B9F25-2435-4A0E-B1D7-79C438C9B06B}"/>
-    <hyperlink ref="G16" r:id="rId64" xr:uid="{4D3D7069-344C-45A1-BA0F-85C18AC6AF01}"/>
-    <hyperlink ref="G18" r:id="rId65" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline Dumbbell Press.webp" xr:uid="{9DA52350-ED9A-4EF0-8D02-735CEAE6526A}"/>
-    <hyperlink ref="G19" r:id="rId66" xr:uid="{0096A054-6DC3-41AE-B284-894E506F0BBA}"/>
-    <hyperlink ref="G23" r:id="rId67" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631394/moveon/Final_Images/Cable Lateral Raises.webp" xr:uid="{06D1FF1C-05AD-497A-B534-19D2AD82B830}"/>
-    <hyperlink ref="G25" r:id="rId68" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631411/moveon/Final_Images/Lateral Raises.webp" xr:uid="{17F90E89-40E1-4697-AC03-D72585511FAC}"/>
-    <hyperlink ref="G31" r:id="rId69" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631411/moveon/Final_Images/Lateral Raises.webp" xr:uid="{F8671347-4C54-40CD-B948-29D2F10A61FB}"/>
-    <hyperlink ref="G28" r:id="rId70" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631390/moveon/Final_Images/Barbell Overhead Press.webp" xr:uid="{FA7CFD3D-A5CA-4E43-9082-A03916DA7967}"/>
-    <hyperlink ref="G29" r:id="rId71" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631394/moveon/Final_Images/Cable Lateral Raises.webp" xr:uid="{06FFE01E-495D-4DC7-B148-9C40681E3619}"/>
-    <hyperlink ref="G30" r:id="rId72" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631400/moveon/Final_Images/Dumbbell Overhead Press.webp" xr:uid="{12EC6382-0ED3-4D62-B7D2-5B31B4A9683D}"/>
-    <hyperlink ref="G32" r:id="rId73" xr:uid="{C92111B9-BB20-495D-9C1B-0D648B62A737}"/>
-    <hyperlink ref="G41" r:id="rId74" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631410/moveon/Final_Images/Lat Pulldowns.webp" xr:uid="{ABBE89A4-9DAB-4338-93E9-03E494A93099}"/>
-    <hyperlink ref="G44" r:id="rId75" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell Rows.webp" xr:uid="{9C959A87-1031-480F-BBA1-778F3612B775}"/>
-    <hyperlink ref="G45" r:id="rId76" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631410/moveon/Final_Images/Lat Pulldowns.webp" xr:uid="{10E58E78-D714-4C6B-81B9-08DD260AEA66}"/>
-    <hyperlink ref="G48" r:id="rId77" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631410/moveon/Final_Images/Lat Pulldowns.webp" xr:uid="{E44A6EDD-EA97-4098-BB8C-4CF43CD40740}"/>
-    <hyperlink ref="G47" r:id="rId78" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631432/moveon/Final_Images/T-Bar Rows.webp" xr:uid="{3C5452B7-2202-4141-9C7A-EC33956810F0}"/>
-    <hyperlink ref="G46" r:id="rId79" xr:uid="{4CD82E2F-A252-445D-9451-8010FD9AD6EB}"/>
-    <hyperlink ref="G49" r:id="rId80" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631427/moveon/Final_Images/Seated Rows Close-Grip.webp" xr:uid="{223B65D7-1449-4DD7-B9F2-5B4A85D2792A}"/>
-    <hyperlink ref="G55" r:id="rId81" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631396/moveon/Final_Images/Concentration Curls.webp" xr:uid="{D01A618E-9222-4F1B-BDF9-091D4164FE77}"/>
-    <hyperlink ref="G56" r:id="rId82" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631389/moveon/Final_Images/Barbell Curls.webp" xr:uid="{50C5EAA6-54A2-4619-8B02-4EDE5AE521AC}"/>
-    <hyperlink ref="G58" r:id="rId83" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631398/moveon/Final_Images/Dumbbell Curls.webp" xr:uid="{39F84755-0259-4DD2-A9FB-D5FEEB83F2EF}"/>
-    <hyperlink ref="G60" r:id="rId84" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631393/moveon/Final_Images/Cable Curls.webp" xr:uid="{F68F2907-CE9C-4ECA-9FED-A239161D66B3}"/>
-    <hyperlink ref="G61" r:id="rId85" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631409/moveon/Final_Images/Incline Dumbbell Curls.webp" xr:uid="{BF6FF696-FF4B-4449-B059-DF08605B4E9D}"/>
-    <hyperlink ref="G64" r:id="rId86" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631433/moveon/Final_Images/Tricep Machine Dip.webp" xr:uid="{AAEA9C6E-5DC5-4D74-9BDF-1FD67822FB35}"/>
-    <hyperlink ref="G69" r:id="rId87" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Rope Pushdowns.webp" xr:uid="{6DCA3703-9DCB-4D07-A0DF-C5D6828151C1}"/>
-    <hyperlink ref="G67" r:id="rId88" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Rope Pushdowns.webp" xr:uid="{46888948-A061-45DC-9F36-DC854A407B92}"/>
-    <hyperlink ref="G71" r:id="rId89" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Rope Pushdowns.webp" xr:uid="{3766BADD-6273-4970-965F-F2BBFF233855}"/>
-    <hyperlink ref="G72" r:id="rId90" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631421/moveon/Final_Images/Rope Pushdowns.webp" xr:uid="{D3C98117-CE42-42A8-B023-2486311396A5}"/>
-    <hyperlink ref="G70" r:id="rId91" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631402/moveon/Final_Images/Dumbbell Tricep Kickback.webp" xr:uid="{5BFA3DE4-9F6D-4BB2-9A1C-5646F8ADE08F}"/>
-    <hyperlink ref="G75" r:id="rId92" xr:uid="{CF4B0320-ADA8-420C-B1C7-459454CB895C}"/>
-    <hyperlink ref="G81" r:id="rId93" xr:uid="{32A749A6-5A70-42B7-9970-CD158C6EE12F}"/>
-    <hyperlink ref="G76" r:id="rId94" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Adductor Machine.webp" xr:uid="{82D2A989-3FC2-49D9-8000-6FB1D1A84AB4}"/>
-    <hyperlink ref="G84" r:id="rId95" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Adductor Machine.webp" xr:uid="{C58B437B-0EA4-46B6-9B12-CE23F2ED7B9C}"/>
-    <hyperlink ref="G90" r:id="rId96" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Adductor Machine.webp" xr:uid="{D948C05A-A122-4E03-9789-57995A381430}"/>
-    <hyperlink ref="G77" r:id="rId97" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Thrust.webp" xr:uid="{221E6130-A9FF-4CE4-9E55-CD3409030E03}"/>
-    <hyperlink ref="G79" r:id="rId98" xr:uid="{7E314C35-C621-4D8A-AF50-0114F3A8AF41}"/>
-    <hyperlink ref="G80" r:id="rId99" xr:uid="{056A179E-C105-4E4E-BB74-9B83D57BDD4F}"/>
-    <hyperlink ref="G83" r:id="rId100" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631425/moveon/Final_Images/Seated Calf Raises.webp" xr:uid="{5E3148BE-8470-47E0-9EAF-04E2CC42377E}"/>
-    <hyperlink ref="G103" r:id="rId101" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631425/moveon/Final_Images/Seated Calf Raises.webp" xr:uid="{3B1903B4-0C3B-4A80-84C9-703D16670551}"/>
-    <hyperlink ref="G78" r:id="rId102" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Standing Calf Raises.webp" xr:uid="{8002D114-BE0B-437F-853C-CE2C1BCDD0ED}"/>
-    <hyperlink ref="G89" r:id="rId103" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Standing Calf Raises.webp" xr:uid="{FA5F2AA2-0574-4639-BC66-82815F98AB29}"/>
-    <hyperlink ref="G107" r:id="rId104" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Standing Calf Raises.webp" xr:uid="{FD242973-F1A5-47EC-8E91-CAA2832DD262}"/>
-    <hyperlink ref="G101" r:id="rId105" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Standing Calf Raises.webp" xr:uid="{3E1DE197-6DF5-487E-BA4D-D10A65ABDB4D}"/>
-    <hyperlink ref="G95" r:id="rId106" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631431/moveon/Final_Images/Standing Calf Raises.webp" xr:uid="{0E89C214-C3C8-4F7F-9D03-2AB8FE0B41B1}"/>
-    <hyperlink ref="G87" r:id="rId107" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631426/moveon/Final_Images/Seated Leg Curl.webp" xr:uid="{400EA336-8AE2-4883-97DC-0F6D7786B52C}"/>
-    <hyperlink ref="G106" r:id="rId108" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631426/moveon/Final_Images/Seated Leg Curl.webp" xr:uid="{A77F8C5B-4FBB-4DD5-89FD-DF0C8A9DFE2E}"/>
-    <hyperlink ref="G96" r:id="rId109" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631407/moveon/Final_Images/Hip Adductor Machine.webp" xr:uid="{6D69030B-D4B1-42A6-BCC0-B66BA24AFE90}"/>
-    <hyperlink ref="G88" r:id="rId110" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631405/moveon/Final_Images/Glute Bridges.webp" xr:uid="{5906C52A-6594-4AAA-8BDE-FEA734C4737B}"/>
-    <hyperlink ref="G99" r:id="rId111" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631412/moveon/Final_Images/Leg Extensions.webp" xr:uid="{77F4402C-BF41-4B51-B987-36870A5AA104}"/>
-    <hyperlink ref="G91" r:id="rId112" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631412/moveon/Final_Images/Leg Extensions.webp" xr:uid="{43130B2B-EDE6-4A5D-A9BA-0D61FA3C00DE}"/>
-    <hyperlink ref="G98" r:id="rId113" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell Squats.webp" xr:uid="{FC3B1F98-6D43-42AF-B735-DFD505C473AC}"/>
-    <hyperlink ref="G104" r:id="rId114" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631391/moveon/Final_Images/Barbell Squats.webp" xr:uid="{319E84B5-F879-4D8A-8626-25EFC478FA27}"/>
-    <hyperlink ref="G93" r:id="rId115" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631413/moveon/Final_Images/Leg Press.webp" xr:uid="{70F9F748-B380-48FB-AC6D-0F1137622CB1}"/>
-    <hyperlink ref="G118" r:id="rId116" display="https://res.cloudinary.com/duprntyar/image/upload/v1776631413/moveon/Final_Images/Leg Raises.webp" xr:uid="{6312C8BB-8557-47E1-A146-ADF49B132BCA}"/>
-    <hyperlink ref="G68" r:id="rId117" xr:uid="{7B36061E-64DF-40F6-9224-B944D441EEE0}"/>
-    <hyperlink ref="G66" r:id="rId118" xr:uid="{642167EC-498A-4DCF-A191-D5E1DD6CD8B2}"/>
-    <hyperlink ref="G114" r:id="rId119" xr:uid="{2DB98109-2989-4E10-B133-D04FC2208178}"/>
+    <hyperlink ref="G3" r:id="rId1" xr:uid="{27C65A5F-CF7E-4784-BF4F-2190B39B3A81}"/>
+    <hyperlink ref="G15" r:id="rId2" xr:uid="{533ED48A-F925-4E26-8045-8E946BA11389}"/>
+    <hyperlink ref="G12" r:id="rId3" xr:uid="{B0B1B76D-A78C-4E35-A325-684A98E0A0B3}"/>
+    <hyperlink ref="G6" r:id="rId4" xr:uid="{CF0C3574-5D85-4BB2-AA65-81FE6058B92D}"/>
+    <hyperlink ref="G9" r:id="rId5" xr:uid="{1507A6EB-2B44-4FA1-A26A-8A702B7BFF8E}"/>
+    <hyperlink ref="G18" r:id="rId6" xr:uid="{761E7FA2-26FE-46C0-8DEB-8C17EB368A35}"/>
+    <hyperlink ref="G22" r:id="rId7" xr:uid="{28EE81CA-AAEF-4AB7-AADF-D1D38410BAFF}"/>
+    <hyperlink ref="G30" r:id="rId8" xr:uid="{767C13B6-CA79-4099-A292-622D72100ACD}"/>
+    <hyperlink ref="G43" r:id="rId9" xr:uid="{D26FF74A-74CA-480C-8D26-9B0AD949720E}"/>
+    <hyperlink ref="G17" r:id="rId10" xr:uid="{897A4AA3-41AC-470C-B7DF-183679F7ABC9}"/>
+    <hyperlink ref="G5" r:id="rId11" xr:uid="{CBD279E5-C94E-44A1-B080-E778BBD674C0}"/>
+    <hyperlink ref="G65" r:id="rId12" xr:uid="{8934AFD0-FA54-4738-A9D1-B65396A275A6}"/>
+    <hyperlink ref="G29" r:id="rId13" xr:uid="{344C1A89-CBF8-4040-8E85-049DF646EFF6}"/>
+    <hyperlink ref="G27" r:id="rId14" xr:uid="{5D058AE7-5FA7-4C64-9B8D-25964ED1983C}"/>
+    <hyperlink ref="G23" r:id="rId15" xr:uid="{5386C541-A8D3-45A1-BB9C-A881AD9747E5}"/>
+    <hyperlink ref="G98" r:id="rId16" xr:uid="{1B6EB5E8-7826-4371-969E-23BC4ED193A4}"/>
+    <hyperlink ref="G92" r:id="rId17" xr:uid="{48E168DF-C6E2-4786-943C-A3E9AED3443E}"/>
+    <hyperlink ref="G117" r:id="rId18" xr:uid="{D699BC8F-6754-4999-A33C-B35CFDCAA1A2}"/>
+    <hyperlink ref="G106" r:id="rId19" xr:uid="{35BB2D92-3104-44E0-84BD-807F67232150}"/>
+    <hyperlink ref="G87" r:id="rId20" xr:uid="{F2A9E9DE-4BAD-404F-B325-5430729F2743}"/>
+    <hyperlink ref="G94" r:id="rId21" xr:uid="{08A2EA39-A64E-42D5-A573-0F41BEA51D92}"/>
+    <hyperlink ref="G10" r:id="rId22" xr:uid="{2CE10C79-782F-42B9-A147-A78257B99802}"/>
+    <hyperlink ref="G64" r:id="rId23" xr:uid="{A8A9156E-D1F0-4032-9768-4AA0930E4CC9}"/>
+    <hyperlink ref="G39" r:id="rId24" xr:uid="{9CD7CA74-BE71-47B3-AEC3-DF44DE87532E}"/>
+    <hyperlink ref="G47" r:id="rId25" xr:uid="{28935E41-1A12-4AAB-B3B9-80B2CD567242}"/>
+    <hyperlink ref="G13" r:id="rId26" xr:uid="{99F30186-D998-4105-A8D1-ED97121E1DF8}"/>
+    <hyperlink ref="G16" r:id="rId27" xr:uid="{1ED23805-F951-407E-B5EC-F1CA2B56E4B9}"/>
+    <hyperlink ref="G19" r:id="rId28" xr:uid="{2DDE6B1D-FB0D-4E82-96E4-B281C56AE287}"/>
+    <hyperlink ref="G59" r:id="rId29" xr:uid="{2B596E3B-D9C7-4B44-B649-F6C978EEB33A}"/>
+    <hyperlink ref="G40" r:id="rId30" xr:uid="{16616CEA-A7D9-45E4-84B2-872D305D818B}"/>
+    <hyperlink ref="G38" r:id="rId31" xr:uid="{DCE255C7-38BE-460A-9C61-B52964DC5635}"/>
+    <hyperlink ref="G46" r:id="rId32" xr:uid="{C3E95146-2D77-4315-8745-9BFC20719B46}"/>
+    <hyperlink ref="G66" r:id="rId33" xr:uid="{FB0D24DA-D365-48BB-91BF-25B0A7C10292}"/>
+    <hyperlink ref="G32" r:id="rId34" xr:uid="{88BBD9D0-D98E-4849-BFBC-D7B6DDA6ADF3}"/>
+    <hyperlink ref="G37" r:id="rId35" xr:uid="{11BC586D-58E1-49AE-B69B-DFB80EFE78BC}"/>
+    <hyperlink ref="G42" r:id="rId36" xr:uid="{E755659A-6014-4095-8217-DCA2232C256D}"/>
+    <hyperlink ref="G53" r:id="rId37" xr:uid="{92FEDF4A-4925-4A76-AB72-5FAE27EEFC81}"/>
+    <hyperlink ref="G24" r:id="rId38" xr:uid="{1228B631-A89E-4BD1-83B6-12A3083D45E2}"/>
+    <hyperlink ref="G63" r:id="rId39" xr:uid="{BED28D9B-BD41-405F-930F-C2F823AD5713}"/>
+    <hyperlink ref="G67" r:id="rId40" xr:uid="{2E1BF5E7-F260-4734-862B-D4DBA991F341}"/>
+    <hyperlink ref="G69" r:id="rId41" xr:uid="{7EEC71A4-5365-4CCC-9D3F-12A631163FD1}"/>
+    <hyperlink ref="G71" r:id="rId42" xr:uid="{1EF061B9-E9B3-41EC-A9E0-DEE1374E794C}"/>
+    <hyperlink ref="G72" r:id="rId43" xr:uid="{7C0E9900-FEBA-4411-8D5E-087BFD28313C}"/>
+    <hyperlink ref="G68" r:id="rId44" xr:uid="{79DE6A30-0D2B-4374-BAD2-63145212EE31}"/>
+    <hyperlink ref="G11" r:id="rId45" xr:uid="{55319F63-2A52-4804-B7BD-B79393DCF255}"/>
+    <hyperlink ref="G8" r:id="rId46" xr:uid="{6CAED313-5282-4171-BDAA-6DBE7BF96D00}"/>
+    <hyperlink ref="G57" r:id="rId47" xr:uid="{63DF1825-BEBB-4C99-9E14-A27004034C8B}"/>
+    <hyperlink ref="G61" r:id="rId48" xr:uid="{29CCC884-8A90-4D88-9100-04ECBCED7238}"/>
+    <hyperlink ref="G25" r:id="rId49" xr:uid="{93DB77A2-968D-4ABD-9F10-629D06EE10E1}"/>
+    <hyperlink ref="G21" r:id="rId50" xr:uid="{1775FC42-9838-4A95-BB4E-CA771DC360B7}"/>
+    <hyperlink ref="G31" r:id="rId51" xr:uid="{B28A69CF-763A-431D-BFF7-ED14B1E99F71}"/>
+    <hyperlink ref="G34" r:id="rId52" xr:uid="{D26BB776-B7BD-4914-93A3-0021ED2BEBEA}"/>
+    <hyperlink ref="G35" r:id="rId53" xr:uid="{BBDDF834-1F20-4390-953C-B7BD89BCFAC3}"/>
+    <hyperlink ref="G41" r:id="rId54" xr:uid="{4318EEC9-F633-4A0E-ACC0-C9F7082552FA}"/>
+    <hyperlink ref="G45" r:id="rId55" xr:uid="{E3CE48D9-DACE-45E7-8D08-B4CB4632A740}"/>
+    <hyperlink ref="G48" r:id="rId56" xr:uid="{B0A11676-B555-4930-A696-B706D207D91D}"/>
+    <hyperlink ref="G26" r:id="rId57" xr:uid="{E82DCF03-706F-41BB-A008-0FFF9992CCCD}"/>
+    <hyperlink ref="G62" r:id="rId58" xr:uid="{90DAEB75-895D-41B3-AAEC-7A400A0CB54B}"/>
+    <hyperlink ref="G70" r:id="rId59" xr:uid="{CBE2F68B-3A36-41A8-B1FD-E64B198BD333}"/>
+    <hyperlink ref="G36" r:id="rId60" xr:uid="{D0454201-F91C-4ECE-9EB8-989F461859B5}"/>
+    <hyperlink ref="G52" r:id="rId61" xr:uid="{F57AB737-6348-4371-B54F-2E4EAE81088E}"/>
+    <hyperlink ref="G58" r:id="rId62" xr:uid="{BA6E58DF-B680-4B24-91F3-BC10F2445399}"/>
+    <hyperlink ref="G73" r:id="rId63" xr:uid="{18397A4B-17C4-4428-AE63-D718EB32E842}"/>
+    <hyperlink ref="G55" r:id="rId64" xr:uid="{51791207-5255-4B13-986D-FCB3B56802EF}"/>
+    <hyperlink ref="G51" r:id="rId65" xr:uid="{B8259CFA-443B-478F-BD7A-88AB6449D218}"/>
+    <hyperlink ref="G2" r:id="rId66" xr:uid="{8C5342FE-46C4-4026-86F6-2ED3C0D956DB}"/>
+    <hyperlink ref="G14" r:id="rId67" xr:uid="{01BE91AB-CCBD-4F60-A55A-A5EB257260C1}"/>
+    <hyperlink ref="G33" r:id="rId68" xr:uid="{54A85FFD-6F17-4AEA-A6CB-E6D7526467F1}"/>
+    <hyperlink ref="G44" r:id="rId69" xr:uid="{F4234217-C062-445F-BCCE-848ECC9E83AB}"/>
+    <hyperlink ref="G54" r:id="rId70" xr:uid="{D39D4638-A763-4BFD-8D3A-C593C48F25A8}"/>
+    <hyperlink ref="G60" r:id="rId71" xr:uid="{8765B606-82FD-44F2-A86E-C43D78D07D41}"/>
+    <hyperlink ref="G50" r:id="rId72" xr:uid="{51EFAE54-B38B-4F64-8015-8C72373B8F43}"/>
+    <hyperlink ref="G56" r:id="rId73" xr:uid="{198E228A-3280-4792-88BB-9040C2A54530}"/>
+    <hyperlink ref="G20" r:id="rId74" xr:uid="{9BF901B5-E9BD-44C8-A3FF-C94E1B7A3A44}"/>
+    <hyperlink ref="G28" r:id="rId75" xr:uid="{C7059C09-D4EF-4C69-8DDE-6DD0C7869DFF}"/>
+    <hyperlink ref="G4" r:id="rId76" xr:uid="{815652AA-80F6-44A3-B3FE-4CCD492B801A}"/>
+    <hyperlink ref="G7" r:id="rId77" xr:uid="{68E7D7B2-112E-409E-860E-D76AC2D4B5D1}"/>
+    <hyperlink ref="G49" r:id="rId78" xr:uid="{9603F9AA-56DF-4B94-8FD4-5B71AA48EC8B}"/>
+    <hyperlink ref="G119" r:id="rId79" xr:uid="{3CFCC7BE-2BB4-4BD3-A56E-7922464EAC9D}"/>
+    <hyperlink ref="G114" r:id="rId80" xr:uid="{735B39EC-370C-4E1D-9BAC-9209D8F06B57}"/>
+    <hyperlink ref="G110" r:id="rId81" xr:uid="{2E32FE7D-F895-4FD0-8D1B-594A550F6B03}"/>
+    <hyperlink ref="G97" r:id="rId82" xr:uid="{010B5F93-43B0-49A6-B407-C4E6B9CAC59D}"/>
+    <hyperlink ref="G88" r:id="rId83" xr:uid="{381ADA21-6CF9-4117-A9AB-825690349ED9}"/>
+    <hyperlink ref="G120" r:id="rId84" xr:uid="{B9BEF9DC-1BA1-4F8B-A7D5-0C6E0548C3A4}"/>
+    <hyperlink ref="G86" r:id="rId85" xr:uid="{68691232-09AB-4D36-B3CC-30332318788D}"/>
+    <hyperlink ref="G115" r:id="rId86" xr:uid="{921EDF11-10CB-40FB-86F2-F5664D5E7F99}"/>
+    <hyperlink ref="G109" r:id="rId87" xr:uid="{FB6C60CC-FEC0-4818-9019-455FF13371E1}"/>
+    <hyperlink ref="G77" r:id="rId88" xr:uid="{CE58C4C4-54FB-45C0-AB01-1E49146ED8E6}"/>
+    <hyperlink ref="G74" r:id="rId89" xr:uid="{49DD6D19-C92E-4904-B2FF-886909DD51F2}"/>
+    <hyperlink ref="G93" r:id="rId90" xr:uid="{38F66F78-06E2-426F-AB49-D53F408A6296}"/>
+    <hyperlink ref="G111" r:id="rId91" xr:uid="{8A4F79DF-D9D4-4C47-B6AC-25D6759F1BEA}"/>
+    <hyperlink ref="G108" r:id="rId92" xr:uid="{5357DE62-42DC-4A9D-88DB-3E9B1EB1E3DD}"/>
+    <hyperlink ref="G102" r:id="rId93" xr:uid="{3CC5813F-E111-467C-81E2-B3D7BAE38F3F}"/>
+    <hyperlink ref="G96" r:id="rId94" xr:uid="{0A04DF87-888A-4AC4-9E31-6C376FB24535}"/>
+    <hyperlink ref="G90" r:id="rId95" xr:uid="{616E528F-1EEE-4741-9CD7-A9B1C50F5F7C}"/>
+    <hyperlink ref="G84" r:id="rId96" xr:uid="{1CC9D3EC-D9AF-481F-A119-F8D335442FFF}"/>
+    <hyperlink ref="G76" r:id="rId97" xr:uid="{397EF8C0-4963-4698-AA06-3F4EA5C33C70}"/>
+    <hyperlink ref="G82" r:id="rId98" xr:uid="{6E5CC3DF-81DA-4E8A-8201-A1E47F458C61}"/>
+    <hyperlink ref="G91" r:id="rId99" xr:uid="{E746A3D7-BF6D-4AEC-A006-2A9394B70AC4}"/>
+    <hyperlink ref="G99" r:id="rId100" xr:uid="{2D6E9E58-14DF-4226-9088-9D4929C66304}"/>
+    <hyperlink ref="G105" r:id="rId101" xr:uid="{F7C362BE-2FFA-4FB7-8A8C-3B1D723C1E36}"/>
+    <hyperlink ref="G79" r:id="rId102" xr:uid="{E137472E-9B01-4E63-ABE4-18B55477A563}"/>
+    <hyperlink ref="G75" r:id="rId103" xr:uid="{BBC921CF-F2F9-4368-B9BA-364D0F184600}"/>
+    <hyperlink ref="G81" r:id="rId104" xr:uid="{1EA5D278-FC74-45AD-82F8-2A58EF1093D9}"/>
+    <hyperlink ref="G100" r:id="rId105" xr:uid="{CA275AA6-DFB3-43C0-AEFE-8FCE7A1B2E86}"/>
+    <hyperlink ref="G116" r:id="rId106" xr:uid="{3AC4A5AC-7471-4933-9C89-31005B6192CB}"/>
+    <hyperlink ref="G112" r:id="rId107" xr:uid="{05A45845-382B-4992-A9A3-D361597A9E48}"/>
+    <hyperlink ref="G85" r:id="rId108" xr:uid="{18EE21C0-724F-4353-84A0-10F2E4AD25C0}"/>
+    <hyperlink ref="G113" r:id="rId109" xr:uid="{6E587F24-30B9-490B-B244-87EAC18F7D85}"/>
+    <hyperlink ref="G103" r:id="rId110" xr:uid="{846D6795-1DBC-48D6-AD4E-4CFE29C720CD}"/>
+    <hyperlink ref="G83" r:id="rId111" xr:uid="{C8D94D2A-D7B5-4B98-9675-EA125D850B58}"/>
+    <hyperlink ref="G80" r:id="rId112" xr:uid="{93B2DD80-D6E8-48E3-9112-85CFF0897B66}"/>
+    <hyperlink ref="G78" r:id="rId113" xr:uid="{71DBA132-A0B2-4559-B887-82045A4F6ED9}"/>
+    <hyperlink ref="G89" r:id="rId114" xr:uid="{028584AF-E47B-4D40-8ED5-2E9F09D94642}"/>
+    <hyperlink ref="G95" r:id="rId115" xr:uid="{82A4421E-5244-4E2C-B394-925B38378299}"/>
+    <hyperlink ref="G101" r:id="rId116" xr:uid="{0A1BA0C9-2AD4-475C-A3C6-9EF77285C20B}"/>
+    <hyperlink ref="G107" r:id="rId117" xr:uid="{85A5240E-9B0C-435A-97BE-BF6D3C36CA0E}"/>
+    <hyperlink ref="G104" r:id="rId118" xr:uid="{C0FF90A4-9080-45CF-9C85-CD1A00897089}"/>
+    <hyperlink ref="G118" r:id="rId119" xr:uid="{07F7D4B1-3250-477E-B237-8CC5FD12BA26}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>